<commit_message>
chore(sweeper): checkpoint 3 dirty path(s)
Automatic additive checkpoint so no work is lost (Standing Rule 29).
Paths were hash-stable for 20s and passed the secret scan.
Top-level areas: build

  build/report-suite/chris-consolidated-2026-08-04

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
+++ b/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
@@ -1459,7 +1459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G164"/>
+  <dimension ref="A1:G165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1486,83 +1486,53 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>NOTE ON NUMBERING: every "item N" INSIDE a carried Source-refs or Resolves cell is the SOURCE SHEET's number, not this workbook's. The "Was" column gives each row's source number. Old -&gt; new: 10-row sheet 1-&gt;Tab 2 item 1, 3-&gt;Tab 2 item 2, 4-&gt;Tab 2 item 3, 5-&gt;Tab 2 item 4, 6-&gt;Tab 2 item 5, 7-&gt;Tab 2 item 6, 8-&gt;Tab 2 item 7, 9-&gt;Tab 2 item 8, 10-&gt;Tab 2 item 9 (its item 2 moved to Tab 1); 17-item sheet 1-&gt;Tab 3 item 1, 2-&gt;Tab 3 item 2, 3-&gt;Tab 3 item 3, 4-&gt;Tab 3 item 4, 5-&gt;Tab 3 item 5, 8-&gt;Tab 3 item 6, 9-&gt;Tab 3 item 7, 10-&gt;Tab 3 item 8, 11-&gt;Tab 3 item 9, 12-&gt;Tab 3 item 10, 14-&gt;Tab 3 item 11, 15-&gt;Tab 3 item 12, 16-&gt;Tab 3 item 13, 17-&gt;Tab 3 item 14 (its items 6, 7 and 13 were de-duplicated out).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Tab</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Was</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Source sheet</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Affected internal case IDs (TestRail C-id)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Spec anchors + live evidence</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>What each answer resolves to</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Tab 1</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>the whole of the one-question sheet</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>chris-location-question-2026-08-04 (the one-question urgent sheet)</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>IV-COL-01 (C30551); IV-COL-04 (C30554); IV-PERS-02 (C30580); IV-EXP-02 (C30588); IV-LOC-06 (C38917); WIP-COL-01 (C30466); WIP-COL-02 (C30467); WIP-FLT-09 (C38916)</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Inventory Value spec v3 S7-R6; WIP spec v6 S4-R3; S7-R13</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>If Chris answers A (automatic - matches both specs): All 8 cases are re-worded to assert the automatic, scope-driven model that SBC/SBR/PV/TU already use, and the observed selector-controlled build is recorded as a DEVIATION in the case notes (the pattern WIP-FLT-05 = C30502 already uses). Two build defects get raised: Work In Progress never shows it automatically; Inventory Value never hides it at single scope on screen. This is the outcome Standing Rule 33 already points to - the specs outrank our build observation - so A costs 8 re-words and 2 tickets. || If Chris answers B (user-toggled): All 8 cases stand exactly as they are; no TestRail write is needed. Chris updates the two written descriptions (WIP S4-R3 + S7-R13, IV S7-R6). The 11 cases on the other four reports that assert the automatic model stay correct, because B would apply only to the two reports whose descriptions change - CONFIRM THIS WITH HIM if he picks B, since a suite-wide B would invalidate those 11. || If Chris answers C (something else / differs per report): Re-derive per report from his answer; expect a further reconciliation pass and treat all 8 as blocked until then. || Regardless of the answer - a separate surface split to settle: On Inventory Value the SCREEN keeps the Location column at single scope while the CSV download drops it (screen observed 2026-08-04; CSV observed 2026-08-03, viu-2026-08-03/evidence/location-matrix/inventory-value__SINGLE__plain.csv has no Location header, __MULTI__ does). Two surfaces, two behaviours - IV-EXP-02 (C30588) is the export case affected. Standing Rule 40: every surface gets its own verdict.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Tab 2</t>
+          <t>Tab 1</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -1572,27 +1542,27 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>item 1 of the 10-row sheet</t>
+          <t>the whole of the one-question sheet</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>chris-sheet-2026-08-04 (the 10-row spec-versus-build sheet)</t>
+          <t>chris-location-question-2026-08-04 (the one-question urgent sheet)</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>SBR-LOC-04 (C30216); PV-FILT-13 (C30340); TU-LOC-05 (C30446); WIP-FLT-06 (C30503); IV-LOC-04 (C30577). NOTE: there is NO Sales By Customer case asserting the hidden filter - SBC-LOC-01 (C30109) only asserts the control's position, so SBC is a coverage question in its own right if he picks B.</t>
+          <t>IV-COL-01 (C30551); IV-COL-04 (C30554); IV-PERS-02 (C30580); IV-EXP-02 (C30588); IV-LOC-06 (C38917); WIP-COL-01 (C30466); WIP-COL-02 (C30467); WIP-FLT-09 (C38916)</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>OUR SOURCE: Chris Ward 2026-07-31 Q1=A, verbatim "A -- classic spec drift" (chris-answers-2026-07-31/answers-ingested.md). THE BUILD'S SOURCE: SBR v15 S21-N1, PV v4 S2-E4, TU v5 S9-N1, IV v3 S7-N1 - all four still read "still sees the filter". LIVE: viu-2026-08-03/evidence/singleloc-matrix.json - hasLocationControl TRUE on all six for the single-workplace subject; build v3.4.1-0ed4433. Verdicts: batch-sbc-sbr/VERDICTS.md SBR-LOC-04, batch-pv-tu/VERDICTS.md PV-FILT-13 + TU-LOC-05, batch-wip-iv/VERDICTS.md IV-LOC-04. RECHECK-QUEUE row B18 (flagged there as the single most important row to re-check).</t>
+          <t>Inventory Value spec v3 S7-R6; WIP spec v6 S4-R3; S7-R13</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>A -&gt; the 5 cases flip from 'filter hidden' to 'filter shown', and SBC needs no new case. B -&gt; no case change; a dev ticket is raised for all six, and SBC needs a NEW case for parity. Either way the four spec notes need his edit. All 5 currently sit DEVIATION and are HELD (batch-wip-iv/STAGED-CHANGES.md group C2) - deliberately not edited, because editing them would assert behaviour no written source supports.</t>
+          <t>If Chris answers A (automatic - matches both specs): All 8 cases are re-worded to assert the automatic, scope-driven model that SBC/SBR/PV/TU already use, and the observed selector-controlled build is recorded as a DEVIATION in the case notes (the pattern WIP-FLT-05 = C30502 already uses). Two build defects get raised: Work In Progress never shows it automatically; Inventory Value never hides it at single scope on screen. This is the outcome Standing Rule 33 already points to - the specs outrank our build observation - so A costs 8 re-words and 2 tickets. || If Chris answers B (user-toggled): All 8 cases stand exactly as they are; no TestRail write is needed. Chris updates the two written descriptions (WIP S4-R3 + S7-R13, IV S7-R6). The 11 cases on the other four reports that assert the automatic model stay correct, because B would apply only to the two reports whose descriptions change - CONFIRM THIS WITH HIM if he picks B, since a suite-wide B would invalidate those 11. || If Chris answers C (something else / differs per report): Re-derive per report from his answer; expect a further reconciliation pass and treat all 8 as blocked until then. || Regardless of the answer - a separate surface split to settle: On Inventory Value the SCREEN keeps the Location column at single scope while the CSV download drops it (screen observed 2026-08-04; CSV observed 2026-08-03, viu-2026-08-03/evidence/location-matrix/inventory-value__SINGLE__plain.csv has no Location header, __MULTI__ does). Two surfaces, two behaviours - IV-EXP-02 (C30588) is the export case affected. Standing Rule 40: every surface gets its own verdict.</t>
         </is>
       </c>
     </row>
@@ -1604,12 +1574,12 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>item 3 of the 10-row sheet</t>
+          <t>item 1 of the 10-row sheet</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -1619,17 +1589,17 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>WIP-COL-05 (C30470); WIP-SORT-03 (C30485); WIP-FLT-03 (C30500); WIP-EXP-07 (C30516). Cross-report reference case, no change proposed: SBC-LBL-01 (C30134).</t>
+          <t>SBR-LOC-04 (C30216); PV-FILT-13 (C30340); TU-LOC-05 (C30446); WIP-FLT-06 (C30503); IV-LOC-04 (C30577). NOTE: there is NO Sales By Customer case asserting the hidden filter - SBC-LOC-01 (C30109) only asserts the control's position, so SBC is a coverage question in its own right if he picks B.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>OUR SOURCE: Chris Ward 2026-07-29, verbatim "A is the correct answer" plus the durable instruction "Not just for these specs though -- really good to keep this in mind for all actions moving forward" (chris-update-2026-07-29/wip-identifier-answer-2026-07-29.md). THE BUILD'S SOURCE: WIP v6 S4-R7 ("the unit number on the first line in bold, and the vehicle identification number on the second line") and S4-R9 ("The Asset column sorts by unit number"). LIVE DOM, verbatim: &lt;div class="wip-asset"&gt;&lt;span class="wip-asset__unit text-weight-bold"&gt;6548&lt;/span&gt;&lt;span class="wip-asset__vin text-caption text-grey-7"&gt;1FDSE3EL1EDB20609&lt;/span&gt;&lt;/div&gt;. Serial-style values live in the VIN field: BULK PARTS1, 12-06696, P631627, 86J8FAC1VALJ43SJY. Build v3.4.1-0ed4433. HONEST LIMIT: we did not CREATE a non-vehicle asset - the report has no asset-creation surface; the terminology point is evidenced from existing records only (batch-wip-iv/STAGED-CHANGES.md group C1).</t>
+          <t>OUR SOURCE: Chris Ward 2026-07-31 Q1=A, verbatim "A -- classic spec drift" (chris-answers-2026-07-31/answers-ingested.md). THE BUILD'S SOURCE: SBR v15 S21-N1, PV v4 S2-E4, TU v5 S9-N1, IV v3 S7-N1 - all four still read "still sees the filter". LIVE: viu-2026-08-03/evidence/singleloc-matrix.json - hasLocationControl TRUE on all six for the single-workplace subject; build v3.4.1-0ed4433. Verdicts: batch-sbc-sbr/VERDICTS.md SBR-LOC-04, batch-pv-tu/VERDICTS.md PV-FILT-13 + TU-LOC-05, batch-wip-iv/VERDICTS.md IV-LOC-04. RECHECK-QUEUE row B18 (flagged there as the single most important row to re-check).</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>A -&gt; dev ticket; the 4 cases stand as written and he edits S4-R7/S4-R9. B -&gt; the 4 cases revert to unit-number-leads and the durable CLAUDE.md ruling is narrowed to exclude this report. C -&gt; a label change is a new question for the whole suite, including SBC-LBL-01. All 4 are HELD, not edited.</t>
+          <t>A -&gt; the 5 cases flip from 'filter hidden' to 'filter shown', and SBC needs no new case. B -&gt; no case change; a dev ticket is raised for all six, and SBC needs a NEW case for parity. Either way the four spec notes need his edit. All 5 currently sit DEVIATION and are HELD (batch-wip-iv/STAGED-CHANGES.md group C2) - deliberately not edited, because editing them would assert behaviour no written source supports.</t>
         </is>
       </c>
     </row>
@@ -1641,12 +1611,12 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>item 4 of the 10-row sheet</t>
+          <t>item 3 of the 10-row sheet</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -1656,17 +1626,17 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>SBR-EXP-10 (C30285); SBR-EXP-11 (C30286).</t>
+          <t>WIP-COL-05 (C30470); WIP-SORT-03 (C30485); WIP-FLT-03 (C30500); WIP-EXP-07 (C30516). Cross-report reference case, no change proposed: SBC-LBL-01 (C30134).</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Three sources, three words. SPEC: SBR v15 S14-R15/S14-R16 both open with `Sales Rep`. OUR SOURCE: Chris Ward 2026-07-31 Q5=A, verbatim "Rep is too much slang, let's do representative everywhere" - so our cases correctly say "Sales Representative" (Rule 32). BUILD: header line read from evidence/location-matrix/sales-by-representative__SINGLE__summary.csv line 2 = `Representative,"Inv. Hrs",...`; the expanded file agrees. Build v3.4.1-0ed4433. Analysis: viu-2026-08-03/LABEL-DIFF.md section A4, which explicitly says do NOT edit these two to "Representative" before he rules.</t>
+          <t>OUR SOURCE: Chris Ward 2026-07-29, verbatim "A is the correct answer" plus the durable instruction "Not just for these specs though -- really good to keep this in mind for all actions moving forward" (chris-update-2026-07-29/wip-identifier-answer-2026-07-29.md). THE BUILD'S SOURCE: WIP v6 S4-R7 ("the unit number on the first line in bold, and the vehicle identification number on the second line") and S4-R9 ("The Asset column sorts by unit number"). LIVE DOM, verbatim: &lt;div class="wip-asset"&gt;&lt;span class="wip-asset__unit text-weight-bold"&gt;6548&lt;/span&gt;&lt;span class="wip-asset__vin text-caption text-grey-7"&gt;1FDSE3EL1EDB20609&lt;/span&gt;&lt;/div&gt;. Serial-style values live in the VIN field: BULK PARTS1, 12-06696, P631627, 86J8FAC1VALJ43SJY. Build v3.4.1-0ed4433. HONEST LIMIT: we did not CREATE a non-vehicle asset - the report has no asset-creation surface; the terminology point is evidenced from existing records only (batch-wip-iv/STAGED-CHANGES.md group C1).</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>A -&gt; both cases reworded to "Representative" and he tidies S14-R15/R16. B -&gt; dev ticket; the cases stand. Either way these two cases also carry item 5 (the four missing columns) and the separate LABEL-DIFF A6 findings (the expanded file puts Invoice # before Date and heads the status column "Invoice Status"), so all of it lands as ONE combined edit per case, each re-verified WHOLE against the current spec per Rule 41.</t>
+          <t>A -&gt; dev ticket; the 4 cases stand as written and he edits S4-R7/S4-R9. B -&gt; the 4 cases revert to unit-number-leads and the durable CLAUDE.md ruling is narrowed to exclude this report. C -&gt; a label change is a new question for the whole suite, including SBC-LBL-01. All 4 are HELD, not edited.</t>
         </is>
       </c>
     </row>
@@ -1678,12 +1648,12 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>item 5 of the 10-row sheet</t>
+          <t>item 4 of the 10-row sheet</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -1693,17 +1663,17 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>SBR-EXP-10 (C30285) - the same case as item 4, so both answers land in one edit.</t>
+          <t>SBR-EXP-10 (C30285); SBR-EXP-11 (C30286).</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>SPEC (Rule 25, verbatim): SBR v15 S14-R15 "Headers, in order: `Sales Rep`, `# Invoices`, `# Customers`, `Hrs Worked`, `Hrs Invoiced`, `Inv. Hrs`, `Labor Invoiced`, `Labor Margin`, `Parts Invoiced`, `Parts Margin`, `Margin`, `Margin %`, `Subtotal`." = 13. BUILD: 9 - `Representative, Inv. Hrs, Labor Invoiced, Labor Margin, Parts Invoiced, Parts Margin, Margin, Margin %, Subtotal` (evidence/location-matrix/sales-by-representative__SINGLE__summary.csv). Missing: # Invoices, # Customers, Hrs Worked, Hrs Invoiced. The payload DOES carry invoice_count, hours_worked and hours_invoiced, which is why LABEL-DIFF.md A5 reads it as an unfinished export, not a data defect. Build v3.4.1-0ed4433. NOTE: S14-R16 itself carries a build note asking engineering to align the hours columns, so his own document already half-anticipates this.</t>
+          <t>Three sources, three words. SPEC: SBR v15 S14-R15/S14-R16 both open with `Sales Rep`. OUR SOURCE: Chris Ward 2026-07-31 Q5=A, verbatim "Rep is too much slang, let's do representative everywhere" - so our cases correctly say "Sales Representative" (Rule 32). BUILD: header line read from evidence/location-matrix/sales-by-representative__SINGLE__summary.csv line 2 = `Representative,"Inv. Hrs",...`; the expanded file agrees. Build v3.4.1-0ed4433. Analysis: viu-2026-08-03/LABEL-DIFF.md section A4, which explicitly says do NOT edit these two to "Representative" before he rules.</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>A -&gt; dev ticket; C30285 stands as written. B -&gt; C30285's enumeration shortens to nine and he shortens S14-R15. Rule 42 applies either way: the rewritten enumeration must carry a version-pinned anchor.</t>
+          <t>A -&gt; both cases reworded to "Representative" and he tidies S14-R15/R16. B -&gt; dev ticket; the cases stand. Either way these two cases also carry item 5 (the four missing columns) and the separate LABEL-DIFF A6 findings (the expanded file puts Invoice # before Date and heads the status column "Invoice Status"), so all of it lands as ONE combined edit per case, each re-verified WHOLE against the current spec per Rule 41.</t>
         </is>
       </c>
     </row>
@@ -1715,12 +1685,12 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>item 6 of the 10-row sheet</t>
+          <t>item 5 of the 10-row sheet</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -1730,17 +1700,17 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>SBC-DATE-01 (C30102); SBC-DATE-03 (C30104) - NOT RUNNABLE TODAY; SBR-DATE-01 (C30201); PV-FILT-03 (C30330); WIP-FLT-04 (C30501); IV-DATE-01 (C30561).</t>
+          <t>SBR-EXP-10 (C30285) - the same case as item 4, so both answers land in one edit.</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>SPEC: SBC v13 S2-R2 closes the eleven-item list verbatim; WIP v6 S7-R6 and IV v3 S5-R1 close the same list in their own words. BUILD: nine presets + inline calendar + "Range: N days" + Apply, captured verbatim in viu-2026-08-03/evidence/date-range-picker.json. Build v3.4.1-0ed4433. This is the application's SHARED date component, so it is a suite-wide product decision. Registered as DELIBERATE-DECISIONS.md entry 2.1 at risk MEDIUM precisely because C30104's steps cannot be executed today.</t>
+          <t>SPEC (Rule 25, verbatim): SBR v15 S14-R15 "Headers, in order: `Sales Rep`, `# Invoices`, `# Customers`, `Hrs Worked`, `Hrs Invoiced`, `Inv. Hrs`, `Labor Invoiced`, `Labor Margin`, `Parts Invoiced`, `Parts Margin`, `Margin`, `Margin %`, `Subtotal`." = 13. BUILD: 9 - `Representative, Inv. Hrs, Labor Invoiced, Labor Margin, Parts Invoiced, Parts Margin, Margin, Margin %, Subtotal` (evidence/location-matrix/sales-by-representative__SINGLE__summary.csv). Missing: # Invoices, # Customers, Hrs Worked, Hrs Invoiced. The payload DOES carry invoice_count, hours_worked and hours_invoiced, which is why LABEL-DIFF.md A5 reads it as an unfinished export, not a data defect. Build v3.4.1-0ed4433. NOTE: S14-R16 itself carries a build note asking engineering to align the hours columns, so his own document already half-anticipates this.</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>A -&gt; 6 cases reworded to the nine presets + calendar, C30104 becomes runnable, and 3 specs need his edit. B -&gt; dev ticket against the shared component; all 6 cases stand and C30104 stays unrunnable until it ships. C -&gt; partial dev ticket plus a partial case rewrite.</t>
+          <t>A -&gt; dev ticket; C30285 stands as written. B -&gt; C30285's enumeration shortens to nine and he shortens S14-R15. Rule 42 applies either way: the rewritten enumeration must carry a version-pinned anchor.</t>
         </is>
       </c>
     </row>
@@ -1752,12 +1722,12 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>item 7 of the 10-row sheet</t>
+          <t>item 6 of the 10-row sheet</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1767,17 +1737,17 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>TU-EXP-01 (C30434); TU-EXP-02 (C30435).</t>
+          <t>SBC-DATE-01 (C30102); SBC-DATE-03 (C30104) - NOT RUNNABLE TODAY; SBR-DATE-01 (C30201); PV-FILT-03 (C30330); WIP-FLT-04 (C30501); IV-DATE-01 (C30561).</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>SPEC (Rule 25, verbatim): TU v5 S7-R2 'an option labeled "Download Summary (PDF)"', S7-R3 '"Download Expanded View (PDF)"', S7-R4 '"Download (CSV)"' = three items with the Download prefix. BUILD: four items - `Summary (PDF)`, `Summary (CSV)`, `Expanded (PDF)`, `Expanded (CSV)`, no prefix (batch-pv-tu/VERDICTS.md TU-EXP-01; evidence/tu/ui/tu-ui-*.json). CONTRAST captured the same run: SBC and SBR both show the four long labels and MATCH their specs exactly (batch-sbc-sbr/VERDICTS.md F2, LABEL-DIFF.md B row SBC-EXP-01). Build v3.4.1-0ed4433. Registered as DELIBERATE-DECISIONS.md entry 2.4, risk MEDIUM.</t>
+          <t>SPEC: SBC v13 S2-R2 closes the eleven-item list verbatim; WIP v6 S7-R6 and IV v3 S5-R1 close the same list in their own words. BUILD: nine presets + inline calendar + "Range: N days" + Apply, captured verbatim in viu-2026-08-03/evidence/date-range-picker.json. Build v3.4.1-0ed4433. This is the application's SHARED date component, so it is a suite-wide product decision. Registered as DELIBERATE-DECISIONS.md entry 2.1 at risk MEDIUM precisely because C30104's steps cannot be executed today.</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>A -&gt; C30434 reworded to the four shipped strings (and C30435's Summary-PDF scope re-checked), and he edits S7-R2/R3/R4 to four items. B -&gt; dev ticket; both cases stand.</t>
+          <t>A -&gt; 6 cases reworded to the nine presets + calendar, C30104 becomes runnable, and 3 specs need his edit. B -&gt; dev ticket against the shared component; all 6 cases stand and C30104 stays unrunnable until it ships. C -&gt; partial dev ticket plus a partial case rewrite.</t>
         </is>
       </c>
     </row>
@@ -1789,12 +1759,12 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>item 8 of the 10-row sheet</t>
+          <t>item 7 of the 10-row sheet</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1804,17 +1774,17 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>IV-EXP-04 (C30590).</t>
+          <t>TU-EXP-01 (C30434); TU-EXP-02 (C30435).</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>SPEC (Rule 25, verbatim): IV v3 S10-R8 "The PDF header shows the report name 'Inventory Value', the organization name, the selected period, and an 'as of' line naming the day the values represent..." - the PDF only; no requirement mentions the CSV. S10-R15 governs only the "Locations:" line. BUILD: CSV line 1 = "As of: 2026-08-03" with the locations line on line 2 (evidence/location-matrix/inventory-value__SINGLE__plain.csv); extracted PDF header block reads `As of 2026-08-04` with NO colon (batch-wip-iv/STAGED-CHANGES.md B28). Build v3.4.1-0ed4433. This surfaced from the SURFACE-MATRIX 1b sweep (Rule 40) - the IV "Locations:" line is the only one of six that is line 2 rather than line 1, because the as-of line sits above it.</t>
+          <t>SPEC (Rule 25, verbatim): TU v5 S7-R2 'an option labeled "Download Summary (PDF)"', S7-R3 '"Download Expanded View (PDF)"', S7-R4 '"Download (CSV)"' = three items with the Download prefix. BUILD: four items - `Summary (PDF)`, `Summary (CSV)`, `Expanded (PDF)`, `Expanded (CSV)`, no prefix (batch-pv-tu/VERDICTS.md TU-EXP-01; evidence/tu/ui/tu-ui-*.json). CONTRAST captured the same run: SBC and SBR both show the four long labels and MATCH their specs exactly (batch-sbc-sbr/VERDICTS.md F2, LABEL-DIFF.md B row SBC-EXP-01). Build v3.4.1-0ed4433. Registered as DELIBERATE-DECISIONS.md entry 2.4, risk MEDIUM.</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>A -&gt; he adds the CSV as-of line to S10-R8 (or a new requirement) and C30590 gains the CSV half. B -&gt; dev ticket to remove it; C30590 unchanged. C -&gt; a wording ticket plus a one-line spec edit; C30590 quotes whichever string he picks.</t>
+          <t>A -&gt; C30434 reworded to the four shipped strings (and C30435's Summary-PDF scope re-checked), and he edits S7-R2/R3/R4 to four items. B -&gt; dev ticket; both cases stand.</t>
         </is>
       </c>
     </row>
@@ -1826,12 +1796,12 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>item 9 of the 10-row sheet</t>
+          <t>item 8 of the 10-row sheet</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1841,17 +1811,17 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>PV-PERM-01 (C30325); PV-PERM-03 (C30327); PV-API-04 (C30391); TU-NAV-07 (C30398); WIP-PERM-01 (C30526); WIP-PERM-02 (C30527); IV-PERM-01 (C30603); IV-PERM-02 (C30604).</t>
+          <t>IV-EXP-04 (C30590).</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>ALREADY RULED - no product decision is being re-asked. Chris Ward 2026-07-31 Q4=A, verbatim "A - the intention is to not hide these from normal reports access. These were specced before CRP was built :)" (and the same answer 2026-07-28), plus the QA LEAD's ruling 2026-08-03, verbatim: "Yes all the reports will be gated by ONE permission FOR NOW." SPEC TEXT STILL STALE: PV v4 S1-R4 + S1-N2, IV v3 Story-1 prerequisite, TU v5 Story-1 prerequisite, WIP v6 Story-1 prerequisite; SBC v13 S1-R2 has been corrected. LIVE PROOF BOTH WAYS (viu-2026-08-03/SURFACE-MATRIX.md Matrix 2 + evidence/permissions/permission-matrix.json + minimal-role-proof.json): the FE permission catalogue holds exactly one report atom; an 8-atom Sales Representative holding only it got 200 on data AND export for all six; a Foreman without it got 403 on all six, data and export. Build v3.4.1-0ed4433. This is why C30327 and C30391 are verified MORE strongly than written - the extra per-report permission does not merely fail to enforce, it does not exist.</t>
+          <t>SPEC (Rule 25, verbatim): IV v3 S10-R8 "The PDF header shows the report name 'Inventory Value', the organization name, the selected period, and an 'as of' line naming the day the values represent..." - the PDF only; no requirement mentions the CSV. S10-R15 governs only the "Locations:" line. BUILD: CSV line 1 = "As of: 2026-08-03" with the locations line on line 2 (evidence/location-matrix/inventory-value__SINGLE__plain.csv); extracted PDF header block reads `As of 2026-08-04` with NO colon (batch-wip-iv/STAGED-CHANGES.md B28). Build v3.4.1-0ed4433. This surfaced from the SURFACE-MATRIX 1b sweep (Rule 40) - the IV "Locations:" line is the only one of six that is line 2 rather than line 1, because the as-of line sits above it.</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>No case change on any answer - all 8 already follow the ruling. This row only closes a documentation debt on four spec pages. The separate rescope-or-retire decision on C30327 and C30391 is the QA LEAD's, not Chris's (chris-answers-2026-08-01/staged-case-plan-CDE-2026-08-03.md).</t>
+          <t>A -&gt; he adds the CSV as-of line to S10-R8 (or a new requirement) and C30590 gains the CSV half. B -&gt; dev ticket to remove it; C30590 unchanged. C -&gt; a wording ticket plus a one-line spec edit; C30590 quotes whichever string he picks.</t>
         </is>
       </c>
     </row>
@@ -1863,12 +1833,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>item 10 of the 10-row sheet</t>
+          <t>item 9 of the 10-row sheet</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1878,54 +1848,54 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>SBC-EXP-01 (C30159); SBC-EXP-14 (C30172).</t>
+          <t>PV-PERM-01 (C30325); PV-PERM-03 (C30327); PV-API-04 (C30391); TU-NAV-07 (C30398); WIP-PERM-01 (C30526); WIP-PERM-02 (C30527); IV-PERM-01 (C30603); IV-PERM-02 (C30604).</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>SPEC: SBC v13 S18-R7 "Exports (CSV, PDF, Print) are generated on the server..." and S18-R10 "If an export (CSV, PDF, or Print) is triggered while the active filters match no customers..." - both still name Print, although Chris retired it in Story 16 ("(removed - Print retired)"). JIRA SV-8614 "SBC - Story 16 - Print the report" is still OPEN. BUILD: a sweep of every button, menu item and link for 'print' in text or aria-label returned an EMPTY list on all six reports (batch-sbc-sbr/VERDICTS.md F3; evidence/sales-by-customer/observe-full.json#toolbar.printControls). Build v3.4.1-0ed4433. Registered as DELIBERATE-DECISIONS.md entry 1.4 at risk LOW, and as an OUTSIDE-IN.md external signal.</t>
+          <t>ALREADY RULED - no product decision is being re-asked. Chris Ward 2026-07-31 Q4=A, verbatim "A - the intention is to not hide these from normal reports access. These were specced before CRP was built :)" (and the same answer 2026-07-28), plus the QA LEAD's ruling 2026-08-03, verbatim: "Yes all the reports will be gated by ONE permission FOR NOW." SPEC TEXT STILL STALE: PV v4 S1-R4 + S1-N2, IV v3 Story-1 prerequisite, TU v5 Story-1 prerequisite, WIP v6 Story-1 prerequisite; SBC v13 S1-R2 has been corrected. LIVE PROOF BOTH WAYS (viu-2026-08-03/SURFACE-MATRIX.md Matrix 2 + evidence/permissions/permission-matrix.json + minimal-role-proof.json): the FE permission catalogue holds exactly one report atom; an 8-atom Sales Representative holding only it got 200 on data AND export for all six; a Foreman without it got 403 on all six, data and export. Build v3.4.1-0ed4433. This is why C30327 and C30391 are verified MORE strongly than written - the extra per-report permission does not merely fail to enforce, it does not exist.</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>No decision and no case change - C30159 explicitly asserts the ABSENCE of Print and PASSED live. Included only so a documentation tidy-up and the closure of SV-8614 are not forgotten; SV-8614 is a dev/ticket action, not Chris's.</t>
+          <t>No case change on any answer - all 8 already follow the ruling. This row only closes a documentation debt on four spec pages. The separate rescope-or-retire decision on C30327 and C30391 is the QA LEAD's, not Chris's (chris-answers-2026-08-01/staged-case-plan-CDE-2026-08-03.md).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Tab 3</t>
+          <t>Tab 2</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>item 1 of the 17-item sheet</t>
+          <t>item 10 of the 10-row sheet</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>PO-Questions-Chris-ReportSuite-2026-08-03 (the 17-item sheet)</t>
+          <t>chris-sheet-2026-08-04 (the 10-row spec-versus-build sheet)</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>SBR-EXP-10 (C30285); SBR-EXP-11 (C30286); SBR-EXP-03 (C30278); SBR-EXP-04 (C30279); SBR-LOC-05 (C38913)</t>
+          <t>SBC-EXP-01 (C30159); SBC-EXP-14 (C30172).</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>SBR spec v15 (Confluence 585629698, lastModified 2026-07-29 - RE-VERIFIED LIVE 2026-08-03, still unresolved): NEW S14-R20 ("included in all four exports in the same position it occupies on screen") vs S14-R15 (Summary CSV headers "in order", beginning `Sales Rep`, no Location) and S14-R16 (Expanded CSV headers). The header enumerations date from the 2026-07-11 "Exports hardened" round and were never amended. Corroborated by contradiction-analysis-2026-07-31/SBR-CSV-LOCATION.md and by Vladimir Tomovic's automated C38923, which was RIGHT (Rule 44).</t>
+          <t>SPEC: SBC v13 S18-R7 "Exports (CSV, PDF, Print) are generated on the server..." and S18-R10 "If an export (CSV, PDF, or Print) is triggered while the active filters match no customers..." - both still name Print, although Chris retired it in Story 16 ("(removed - Print retired)"). JIRA SV-8614 "SBC - Story 16 - Print the report" is still OPEN. BUILD: a sweep of every button, menu item and link for 'print' in text or aria-label returned an EMPTY list on all six reports (batch-sbc-sbr/VERDICTS.md F3; evidence/sales-by-customer/observe-full.json#toolbar.printControls). Build v3.4.1-0ed4433. Registered as DELIBERATE-DECISIONS.md entry 1.4 at risk LOW, and as an OUTSIDE-IN.md external signal.</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>A -&gt; the 5 cases stand as pushed and Chris tidies S14-R15/R16. B -&gt; revert the export halves to the fixed lists and drop the Location assertions. Same on-screen/export split was fixed on SBC (S4-R13), PV (S6-R11), TU (S7-R13), IV (S10-R15); WIP already had it. Either way VIU-confirm live.</t>
+          <t>No decision and no case change - C30159 explicitly asserts the ABSENCE of Print and PASSED live. Included only so a documentation tidy-up and the closure of SV-8614 are not forgotten; SV-8614 is a dev/ticket action, not Chris's.</t>
         </is>
       </c>
     </row>
@@ -1937,12 +1907,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>item 2 of the 17-item sheet</t>
+          <t>item 1 of the 17-item sheet</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1952,17 +1922,17 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>WIP-COL-05 (C30470); WIP-FLT-03 (C30500); WIP-SORT-03 (C30485); WIP-EXP-07 (C30516); SBR-LOC-04 (C30216); TU-LOC-05 (C30446); IV-LOC-04 (C30577); PV-FILT-13 (C30340); TU-NAV-01 (C30392); PV-NAV-01 (C30322)</t>
+          <t>SBR-EXP-10 (C30285); SBR-EXP-11 (C30286); SBR-EXP-03 (C30278); SBR-EXP-04 (C30279); SBR-LOC-05 (C38913)</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>SPEC-WATCH-2026-07-28.md re-diff 2026-07-31, re-confirmed 2026-08-03 (all five non-SBC specs still at their 2026-07-29 versions per live CQL, so nothing has landed since): 7 of 12 items still need spec text - 1b WIP identifier, 4 location filter hidden, 6 nav placement wording, 8 WIP asset dropdown, 9 customer-card Representative, 10 SBC nav anchors, 11 PV "only report". Deadline 2026-08-04.</t>
+          <t>SBR spec v15 (Confluence 585629698, lastModified 2026-07-29 - RE-VERIFIED LIVE 2026-08-03, still unresolved): NEW S14-R20 ("included in all four exports in the same position it occupies on screen") vs S14-R15 (Summary CSV headers "in order", beginning `Sales Rep`, no Location) and S14-R16 (Expanded CSV headers). The header enumerations date from the 2026-07-11 "Exports hardened" round and were never amended. Corroborated by contradiction-analysis-2026-07-31/SBR-CSV-LOCATION.md and by Vladimir Tomovic's automated C38923, which was RIGHT (Rule 44).</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>A -&gt; no case change; SPEC-WATCH stays open until the text lands. B -&gt; SPEC-WATCH closes as a documentation debt. Neither answer changes a case. Items 1b/4/6/9/10/11 are ALSO asked individually as sheet items 6-12 so he can tick them off.</t>
+          <t>A -&gt; the 5 cases stand as pushed and Chris tidies S14-R15/R16. B -&gt; revert the export halves to the fixed lists and drop the Location assertions. Same on-screen/export split was fixed on SBC (S4-R13), PV (S6-R11), TU (S7-R13), IV (S10-R15); WIP already had it. Either way VIU-confirm live.</t>
         </is>
       </c>
     </row>
@@ -1974,12 +1944,12 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>item 3 of the 17-item sheet</t>
+          <t>item 2 of the 17-item sheet</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1989,17 +1959,17 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>SBC-EXP-16 (C38856); SBC-LOC-04 (C38912); SBR-EXP-10 (C30285); SBR-EXP-03 (C30278); SBR-LOC-05 (C38913)</t>
+          <t>WIP-COL-05 (C30470); WIP-FLT-03 (C30500); WIP-SORT-03 (C30485); WIP-EXP-07 (C30516); SBR-LOC-04 (C30216); TU-LOC-05 (C30446); IV-LOC-04 (C30577); PV-FILT-13 (C30340); TU-NAV-01 (C30392); PV-NAV-01 (C30322)</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>SPEC-SILENT, found by coverage-rederivation-2026-07-31. SBC S4-R13 states inclusion with no position; SBR S14-R20 says "the same position it occupies on screen" but the Summary CSV (S14-R15) has no Date/Status column and the Summary PDF (S14-R5) has none either. Cases currently hedge ("with the identifying columns ahead of the money columns (confirm its exact position in the build)") - hedged, not invented (Rule 9).</t>
+          <t>SPEC-WATCH-2026-07-28.md re-diff 2026-07-31, re-confirmed 2026-08-03 (all five non-SBC specs still at their 2026-07-29 versions per live CQL, so nothing has landed since): 7 of 12 items still need spec text - 1b WIP identifier, 4 location filter hidden, 6 nav placement wording, 8 WIP asset dropdown, 9 customer-card Representative, 10 SBC nav anchors, 11 PV "only report". Deadline 2026-08-04.</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>A -&gt; replace the hedge with the stated position. B -&gt; reword to far-right. C -&gt; keep the hedge and pin it at VIU. No case is wrong today either way.</t>
+          <t>A -&gt; no case change; SPEC-WATCH stays open until the text lands. B -&gt; SPEC-WATCH closes as a documentation debt. Neither answer changes a case. Items 1b/4/6/9/10/11 are ALSO asked individually as sheet items 6-12 so he can tick them off.</t>
         </is>
       </c>
     </row>
@@ -2011,12 +1981,12 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>item 4 of the 17-item sheet</t>
+          <t>item 3 of the 17-item sheet</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -2026,17 +1996,17 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>SBC-EXP-10 (C30168); TU-EXP-06 (C30439); TU-EXP-07 (C30440); PV-EXP-05 (C30379); PV-EXP-06 (C30380); SBR-EXP-03 (C30278); SBR-EXP-04 (C30279)</t>
+          <t>SBC-EXP-16 (C38856); SBC-LOC-04 (C38912); SBR-EXP-10 (C30285); SBR-EXP-03 (C30278); SBR-LOC-05 (C38913)</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Cross-report spec contradiction against his 2026-07-29 message ("Each report now ensures the same 'logo' treatment"): SBC S15-R16/R17/R18 = 3-step chain ending in NO logo; TU = bundled ShopView default; PV has no logo requirement at all. DELIBERATE-DECISIONS.md A2. Not resolved by us (Rule 15 - never pick a side silently).</t>
+          <t>SPEC-SILENT, found by coverage-rederivation-2026-07-31. SBC S4-R13 states inclusion with no position; SBR S14-R20 says "the same position it occupies on screen" but the Summary CSV (S14-R15) has no Date/Status column and the Summary PDF (S14-R5) has none either. Cases currently hedge ("with the identifying columns ahead of the money columns (confirm its exact position in the build)") - hedged, not invented (Rule 9).</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>A -&gt; TU/PV export cases gain the fallback chain. B -&gt; SBC-EXP-10's chain collapses to the bundled default. C -&gt; re-ask. Wording-only edits either way.</t>
+          <t>A -&gt; replace the hedge with the stated position. B -&gt; reword to far-right. C -&gt; keep the hedge and pin it at VIU. No case is wrong today either way.</t>
         </is>
       </c>
     </row>
@@ -2048,12 +2018,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>item 5 of the 17-item sheet</t>
+          <t>item 4 of the 17-item sheet</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -2063,17 +2033,17 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>NONE - zero case impact either way. Evidence base: SBC-DATE-01 (C30102) asserts the ABSENCE of "All Time"; the SBC Print case was retired 2026-07-28 (deleted from TestRail, so it has no live C-id); no case exists for customer comparison, asset comparison or global-search narrowing</t>
+          <t>SBC-EXP-10 (C30168); TU-EXP-06 (C30439); TU-EXP-07 (C30440); PV-EXP-05 (C30379); PV-EXP-06 (C30380); SBR-EXP-03 (C30278); SBR-EXP-04 (C30279)</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>His chat, verbatim: "SBC actually has several features that we dropped almost right before the squad assembled ... the requirements should have dropped with the additional features dropping, I own that." Checked live 2026-08-03 against the SBC spec change log (Confluence 577634305): the four dropped rounds are 2026-07-12 (customer comparison + asset comparison), 2026-07-15 (global search), 2026-07-16 (All Time), 2026-07-29 (Print). ZERO lingering requirements and ZERO stale cases found - see chris-answers-2026-08-01/answers-ingested.md section 3.</t>
+          <t>Cross-report spec contradiction against his 2026-07-29 message ("Each report now ensures the same 'logo' treatment"): SBC S15-R16/R17/R18 = 3-step chain ending in NO logo; TU = bundled ShopView default; PV has no logo requirement at all. DELIBERATE-DECISIONS.md A2. Not resolved by us (Rule 15 - never pick a side silently).</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>A -&gt; the item closes with a written all-clear. B -&gt; re-derive coverage for whatever he names. We did NOT manufacture a retire list to fill the gap (Rule 12).</t>
+          <t>A -&gt; TU/PV export cases gain the fallback chain. B -&gt; SBC-EXP-10's chain collapses to the bundled default. C -&gt; re-ask. Wording-only edits either way.</t>
         </is>
       </c>
     </row>
@@ -2085,12 +2055,12 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>item 8 of the 17-item sheet</t>
+          <t>item 5 of the 17-item sheet</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -2100,17 +2070,17 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off</t>
+          <t>NONE - zero case impact either way. Evidence base: SBC-DATE-01 (C30102) asserts the ABSENCE of "All Time"; the SBC Print case was retired 2026-07-28 (deleted from TestRail, so it has no live C-id); no case exists for customer comparison, asset comparison or global-search narrowing</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>Named individually at the QA lead's instruction ("each named individually, not as a bundle"), because the 2026-08-04 deadline is tomorrow and a bundled question has so far produced a bundled non-answer. [this mapping row covers items 6-12 of the source sheet; after the de-duplication its surviving items are Tab 3 items 6, 7, 8, 9, 10]</t>
+          <t>His chat, verbatim: "SBC actually has several features that we dropped almost right before the squad assembled ... the requirements should have dropped with the additional features dropping, I own that." Checked live 2026-08-03 against the SBC spec change log (Confluence 577634305): the four dropped rounds are 2026-07-12 (customer comparison + asset comparison), 2026-07-15 (global search), 2026-07-16 (All Time), 2026-07-29 (Print). ZERO lingering requirements and ZERO stale cases found - see chris-answers-2026-08-01/answers-ingested.md section 3.</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>No case change on any answer - the cases already follow his rulings (Rule 32). These only close a documentation debt.</t>
+          <t>A -&gt; the item closes with a written all-clear. B -&gt; re-derive coverage for whatever he names. We did NOT manufacture a retire list to fill the gap (Rule 12).</t>
         </is>
       </c>
     </row>
@@ -2122,12 +2092,12 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>item 9 of the 17-item sheet</t>
+          <t>item 8 of the 17-item sheet</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -2137,7 +2107,7 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off</t>
+          <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off ["row 2" here means the source sheet's own item-2 mapping row, which is Tab 3 item 2 above]</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -2159,12 +2129,12 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>item 10 of the 17-item sheet</t>
+          <t>item 9 of the 17-item sheet</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -2174,7 +2144,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off</t>
+          <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off ["row 2" here means the source sheet's own item-2 mapping row, which is Tab 3 item 2 above]</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -2196,12 +2166,12 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>item 11 of the 17-item sheet</t>
+          <t>item 10 of the 17-item sheet</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2211,7 +2181,7 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off</t>
+          <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off ["row 2" here means the source sheet's own item-2 mapping row, which is Tab 3 item 2 above]</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -2233,12 +2203,12 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>item 12 of the 17-item sheet</t>
+          <t>item 11 of the 17-item sheet</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -2248,7 +2218,7 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off</t>
+          <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off ["row 2" here means the source sheet's own item-2 mapping row, which is Tab 3 item 2 above]</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
@@ -2270,12 +2240,12 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>item 14 of the 17-item sheet</t>
+          <t>item 12 of the 17-item sheet</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2285,17 +2255,17 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>SBR-DEACT-04 (C30255)</t>
+          <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off ["row 2" here means the source sheet's own item-2 mapping row, which is Tab 3 item 2 above]</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>ANSWERED by Chris 2026-07-28, verbatim "B." (chris-answers-2026-07-28/answers-ingested.md Q1) = Escape must NOT dismiss. Verified live 2026-08-03: SBR S13-R8 still says Escape closes the dialog. NOTE - a correction to our own record: PO-Questions-Chris-ReportSuite-2026-07-31.md line 125 says this question is still "open four days". That is STALE; only the spec text remains outstanding, which is why this appears here as a write-down item, not a decision.</t>
+          <t>Named individually at the QA lead's instruction ("each named individually, not as a bundle"), because the 2026-08-04 deadline is tomorrow and a bundled question has so far produced a bundled non-answer. [this mapping row covers items 6-12 of the source sheet; after the de-duplication its surviving items are Tab 3 items 6, 7, 8, 9, 10]</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>No case change - C30255 already follows his answer.</t>
+          <t>No case change on any answer - the cases already follow his rulings (Rule 32). These only close a documentation debt.</t>
         </is>
       </c>
     </row>
@@ -2307,12 +2277,12 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>item 15 of the 17-item sheet</t>
+          <t>item 14 of the 17-item sheet</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -2322,17 +2292,17 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>PV-EXP-11 (C38885); TU-EXP-09 (C38887); WIP-EXP-10 (C38918)</t>
+          <t>SBR-DEACT-04 (C30255)</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>His 2026-07-31 Q2=A ("A - great catch", one suite-wide message) + Q3=A ("this was not well thought out by me", cap on all six). Verified: the PV/TU/WIP pages carry no cap line; the three cases exist and are pushed.</t>
+          <t>ANSWERED by Chris 2026-07-28, verbatim "B." (chris-answers-2026-07-28/answers-ingested.md Q1) = Escape must NOT dismiss. Verified live 2026-08-03: SBR S13-R8 still says Escape closes the dialog. NOTE - a correction to our own record: PO-Questions-Chris-ReportSuite-2026-07-31.md line 125 says this question is still "open four days". That is STALE; only the spec text remains outstanding, which is why this appears here as a write-down item, not a decision.</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>No case change - documentation debt only.</t>
+          <t>No case change - C30255 already follows his answer.</t>
         </is>
       </c>
     </row>
@@ -2344,12 +2314,12 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>12</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>item 16 of the 17-item sheet</t>
+          <t>item 15 of the 17-item sheet</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -2359,17 +2329,17 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>SBC-LBL-01 (C30134); WIP-COL-05 (C30470)</t>
+          <t>PV-EXP-11 (C38885); TU-EXP-09 (C38887); WIP-EXP-10 (C38918)</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>His own 2026-07-29 standing note, verbatim: "we just have to be careful with using the acronym VIN ... for a generator ... it gets confusing". Our cases keep the build label "VIN" plus a plain tester note, per the durable ruling in CLAUDE.md.</t>
+          <t>His 2026-07-31 Q2=A ("A - great catch", one suite-wide message) + Q3=A ("this was not well thought out by me", cap on all six). Verified: the PV/TU/WIP pages carry no cap line; the three cases exist and are pushed.</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>No case change either way - the on-screen label is unaffected.</t>
+          <t>No case change - documentation debt only.</t>
         </is>
       </c>
     </row>
@@ -2381,121 +2351,126 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>item 16 of the 17-item sheet</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>PO-Questions-Chris-ReportSuite-2026-08-03 (the 17-item sheet)</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>SBC-LBL-01 (C30134); WIP-COL-05 (C30470)</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>His own 2026-07-29 standing note, verbatim: "we just have to be careful with using the acronym VIN ... for a generator ... it gets confusing". Our cases keep the build label "VIN" plus a plain tester note, per the durable ruling in CLAUDE.md.</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>No case change either way - the on-screen label is unaffected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Tab 3</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
           <t>14</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>item 17 of the 17-item sheet</t>
         </is>
       </c>
-      <c r="D28" s="6" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>PO-Questions-Chris-ReportSuite-2026-08-03 (the 17-item sheet)</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>NONE</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
         <is>
           <t>Cosmetic encoding artefact (mojibake) in the SBR and PV spec text, already noted in SPEC-WATCH-2026-07-28.md. Not a product question; asked only because it makes quoting those lines back to him unreliable.</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>No case impact.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>THE LINKS, SPELLED OUT (Tab 1's eight cases)</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Internal ID</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>TestRail C-id</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>Report</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>Spec anchor</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="F32" s="3" t="inlineStr">
         <is>
           <t>What it asserts today</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>IV-COL-01</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>C30551</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30551</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>Inventory Value</t>
-        </is>
-      </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>Inventory Value spec v3 S7-R6</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>Asserts Location is in the column-selection control and appears 'when it is turned on', between Vendor and Qty.</t>
-        </is>
-      </c>
+      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>IV-COL-04</t>
+          <t>IV-COL-01</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>C30554</t>
+          <t>C30551</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30554</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30551</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -2510,24 +2485,24 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>Asserts Location can be 'turned on from the column-selection control' and then appears in its fixed position.</t>
+          <t>Asserts Location is in the column-selection control and appears 'when it is turned on', between Vendor and Qty.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>IV-PERS-02</t>
+          <t>IV-COL-04</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>C30580</t>
+          <t>C30554</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30580</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30554</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -2542,24 +2517,24 @@
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>Fixed column order stated 'with Location, when it is turned on in the column-selection control, between Vendor and Qty'.</t>
+          <t>Asserts Location can be 'turned on from the column-selection control' and then appears in its fixed position.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>IV-EXP-02</t>
+          <t>IV-PERS-02</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>C30588</t>
+          <t>C30580</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30588</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30580</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
@@ -2574,24 +2549,24 @@
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>Tester note says the files carry Location 'when Location is turned ON in the column-selection control'.</t>
+          <t>Fixed column order stated 'with Location, when it is turned on in the column-selection control, between Vendor and Qty'.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>IV-LOC-06</t>
+          <t>IV-EXP-02</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>C38917</t>
+          <t>C30588</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/38917</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30588</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
@@ -2606,56 +2581,56 @@
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>Step 1 instructs the tester to 'Turn Location on in the column-selection control'; expected says visibility 'follows that toggle, not the location selection'.</t>
+          <t>Tester note says the files carry Location 'when Location is turned ON in the column-selection control'.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>WIP-COL-01</t>
+          <t>IV-LOC-06</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>C30466</t>
+          <t>C38917</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30466</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/38917</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Work In Progress</t>
+          <t>Inventory Value</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>WIP spec v6 S4-R3; S7-R13</t>
+          <t>Inventory Value spec v3 S7-R6</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>Precondition 4: 'Location is turned ON in the column-selection control (it is off by default).'</t>
+          <t>Step 1 instructs the tester to 'Turn Location on in the column-selection control'; expected says visibility 'follows that toggle, not the location selection'.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>WIP-COL-02</t>
+          <t>WIP-COL-01</t>
         </is>
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>C30467</t>
+          <t>C30466</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/30467</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30466</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -2670,270 +2645,270 @@
       </c>
       <c r="F38" s="6" t="inlineStr">
         <is>
-          <t>Asserts Location IS offered in the selector, off by default, and does 'NOT appear on its own' - and says out loud 'That is what the build does today.'</t>
+          <t>Precondition 4: 'Location is turned ON in the column-selection control (it is off by default).'</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
+          <t>WIP-COL-02</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>C30467</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30467</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>Work In Progress</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>WIP spec v6 S4-R3; S7-R13</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>Asserts Location IS offered in the selector, off by default, and does 'NOT appear on its own' - and says out loud 'That is what the build does today.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
           <t>WIP-FLT-09</t>
         </is>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>C38916</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/38916</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>Work In Progress</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>WIP spec v6 S4-R3; S7-R13</t>
         </is>
       </c>
-      <c r="F39" s="6" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>Asserts 'The column does not appear or disappear on its own ... it follows the column-selection toggle only.'</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="1" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
         <is>
           <t>DE-DUPLICATION LOG - 4 OVERLAPPING ITEMS REMOVED (28 IN, 24 OUT)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>Removed</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>The item</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr">
         <is>
           <t>What happened</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr">
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>Why, and what was preserved</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>Tab 2, item 2 of the 10-row sheet</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="inlineStr">
-        <is>
-          <t>"The extra location column works one way on Work In Progress and the exact opposite way on Inventory Value"</t>
-        </is>
-      </c>
-      <c r="C43" s="6" t="inlineStr">
-        <is>
-          <t>REMOVED — the same question, asked wider, is Tab 1</t>
-        </is>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>Tab 1 asks the identical question (automatic versus a switch the user controls) but across all SIX reports and adds the screen-versus-download split on Inventory Value, so it is the superset. Asking both would have let him answer the two-report version and the six-report version differently. Its QA mapping row is RETAINED below — it carries WIP-PERS-02 (C30507), which Tab 1's own eight-case list does not.</t>
-        </is>
-      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>Tab 3, item 6 of the 17-item sheet</t>
+          <t>Tab 2, item 2 of the 10-row sheet</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>"Work In Progress: which number identifies the vehicle or machine first" — will you update the description?</t>
+          <t>"The extra location column works one way on Work In Progress and the exact opposite way on Inventory Value"</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>REMOVED — subsumed by Tab 2 item 3</t>
+          <t>REMOVED - the same question, asked wider, is Tab 1</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>Tab 2 item 3 asks which side moves now the product disagrees with his 29 July ruling, and BOTH of its options already name who edits the write-up. Keeping the separate tick-box allowed a contradiction: he could tick "yes I will update it" here and choose "keep the product as it is" there. Its QA mapping row is RETAINED below.</t>
+          <t>Tab 1 asks the identical question (automatic versus a switch the user controls) but across all SIX reports and adds the screen-versus-download split on Inventory Value, so it is the superset. Asking both would have let him answer the two-report version and the six-report version differently. Its QA mapping row is RETAINED below - it carries WIP-PERS-02 (C30507), which Tab 1's own eight-case list does not.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>Tab 3, item 7 of the 17-item sheet</t>
+          <t>Tab 3, item 6 of the 17-item sheet</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>"The location chooser is hidden for someone with only one location" — will you correct those four lines?</t>
+          <t>"Work In Progress: which number identifies the vehicle or machine first" - will you update the description?</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>REMOVED — subsumed by Tab 2 item 1</t>
+          <t>REMOVED - subsumed by Tab 2 item 2</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>Tab 2 item 1 puts the same four quoted lines in front of him and says in BOTH options that the four lines need correcting. Same contradiction risk as above. Its QA mapping row is RETAINED below.</t>
+          <t>Tab 2 item 2 asks which side moves now the product disagrees with his 29 July ruling, and BOTH of its options already name who edits the write-up. Keeping the separate tick-box allowed a contradiction: he could tick "yes I will update it" here and choose "keep the product as it is" there. Its QA mapping row is RETAINED below.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
+          <t>Tab 3, item 7 of the 17-item sheet</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>"The location chooser is hidden for someone with only one location" - will you correct those four lines?</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>REMOVED - subsumed by Tab 2 item 1</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>Tab 2 item 1 puts the same four quoted lines in front of him and says in BOTH options that the four lines need correcting. Same contradiction risk as above. Its QA mapping row is RETAINED below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
           <t>Tab 3, item 13 of the 17-item sheet</t>
         </is>
       </c>
-      <c r="B46" s="6" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>"Five descriptions still say the report needs its own area permission"</t>
         </is>
       </c>
-      <c r="C46" s="6" t="inlineStr">
-        <is>
-          <t>REMOVED — exact duplicate of Tab 2 item 9</t>
-        </is>
-      </c>
-      <c r="D46" s="6" t="inlineStr">
-        <is>
-          <t>The 10-row sheet already recorded this as the one overlap between the two sheets. Tab 2's version is the better one: it carries the live both-ways proof, and its figure is right — it says FOUR write-ups and lists four, whereas this row said "five" and then listed four. So the removal also retires a stale figure. Its QA mapping row is RETAINED below — it carries four navigation/tab cases (PV-NAV-01, IV-NAV-01, TU-NAV-01, WIP-TAB-01) that Tab 2 item 9's row does not.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="1" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>REMOVED - exact duplicate of Tab 2 item 8</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>The 10-row sheet already recorded this as the one overlap between the two sheets. Tab 2's version is the better one: it carries the live both-ways proof, and its figure is right - it says FOUR write-ups and lists four, whereas this row said "five" and then listed four. So the removal also retires a stale figure. Its QA mapping row is RETAINED below - it carries four navigation/tab cases (PV-NAV-01, IV-NAV-01, TU-NAV-01, WIP-TAB-01) that Tab 2 item 8's row does not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
         <is>
           <t>MERGED OUT - THE REMOVED ITEMS' QA MAPPING ROWS, RETAINED SO NO CASE ID IS LOST</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
         <is>
           <t>Was</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Source sheet</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr">
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>Now asked as</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>Affected internal case IDs (TestRail C-id)</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E50" s="3" t="inlineStr">
         <is>
           <t>Spec anchors + live evidence</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="F50" s="3" t="inlineStr">
         <is>
           <t>What each answer resolves to</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>item 2 of the 10-row sheet</t>
-        </is>
-      </c>
-      <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>chris-sheet-2026-08-04 (the 10-row spec-versus-build sheet)</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>asked once, as Tab 1</t>
-        </is>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>Work In Progress: WIP-COL-02 (C30467); WIP-COL-01 (C30466); WIP-PERS-02 (C30507); WIP-FLT-09 (C38916). Inventory Value: IV-LOC-06 (C38917); IV-COL-04 (C30554).</t>
-        </is>
-      </c>
-      <c r="E50" s="6" t="inlineStr">
-        <is>
-          <t>SPEC: WIP v6 S4-R3 + S7-R13 ("not offered in the column selector; its visibility is automatic"); IV v3 Story-7 context note + S7-R7 ("not a user-toggled column in the column-selection control"). LIVE: viu-2026-08-03/batch-wip-iv/evidence/ui/colsel-work-in-progress.json - Location is item index 5 of 16, ariaChecked=false; colsel-inventory-value.json - Location is item index 4 of 11, ariaChecked=true; iv-singleloc.png shows the column still present with the chooser narrowed to Staging Lethbridge - 4310. Build v3.4.1-0ed4433. ALSO OUR OWN CONTRADICTION (Rule 28 cross-case sweep): C30466 and C30507 both list Location inside the toggleable order while C30467 says it is not offered - that self-contradiction is resolved whichever way he rules. HONEST LIMIT: the separate one-location-USER read of the IV screen was CONFOUNDED by a persisted column selection (RECHECK-QUEUE B34, recorded NOT VERIFIED); the observation quoted to Chris is the ADMIN-NARROWING one, which is clean. Note also that the IV single-location CSV has NO Location column (evidence/location-matrix/inventory-value__SINGLE__plain.csv), so the download already follows the automatic rule while the screen follows the toggle.</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>A -&gt; dev ticket for both reports; the 6 cases stand as written and the two specs need no change. B -&gt; both specs need his edit and the 6 cases are reworded to the toggle model (WIP off-by-default, IV on-by-default, or one agreed default). C -&gt; the two reports are documented as deliberately different and our cross-case contradiction is closed by writing each report's own model down.</t>
-        </is>
-      </c>
+      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>item 6 of the 17-item sheet</t>
+          <t>item 2 of the 10-row sheet</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>PO-Questions-Chris-ReportSuite-2026-08-03 (the 17-item sheet)</t>
+          <t>chris-sheet-2026-08-04 (the 10-row spec-versus-build sheet)</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>asked once, as Tab 2 item 3</t>
+          <t>asked once, as Tab 1</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off</t>
+          <t>Work In Progress: WIP-COL-02 (C30467); WIP-COL-01 (C30466); WIP-PERS-02 (C30507); WIP-FLT-09 (C38916). Inventory Value: IV-LOC-06 (C38917); IV-COL-04 (C30554).</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>Named individually at the QA lead's instruction ("each named individually, not as a bundle"), because the 2026-08-04 deadline is tomorrow and a bundled question has so far produced a bundled non-answer.</t>
+          <t>SPEC: WIP v6 S4-R3 + S7-R13 ("not offered in the column selector; its visibility is automatic"); IV v3 Story-7 context note + S7-R7 ("not a user-toggled column in the column-selection control"). LIVE: viu-2026-08-03/batch-wip-iv/evidence/ui/colsel-work-in-progress.json - Location is item index 5 of 16, ariaChecked=false; colsel-inventory-value.json - Location is item index 4 of 11, ariaChecked=true; iv-singleloc.png shows the column still present with the chooser narrowed to Staging Lethbridge - 4310. Build v3.4.1-0ed4433. ALSO OUR OWN CONTRADICTION (Rule 28 cross-case sweep): C30466 and C30507 both list Location inside the toggleable order while C30467 says it is not offered - that self-contradiction is resolved whichever way he rules. HONEST LIMIT: the separate one-location-USER read of the IV screen was CONFOUNDED by a persisted column selection (RECHECK-QUEUE B34, recorded NOT VERIFIED); the observation quoted to Chris is the ADMIN-NARROWING one, which is clean. Note also that the IV single-location CSV has NO Location column (evidence/location-matrix/inventory-value__SINGLE__plain.csv), so the download already follows the automatic rule while the screen follows the toggle.</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>No case change on any answer - the cases already follow his rulings (Rule 32). These only close a documentation debt.</t>
+          <t>A -&gt; dev ticket for both reports; the 6 cases stand as written and the two specs need no change. B -&gt; both specs need his edit and the 6 cases are reworded to the toggle model (WIP off-by-default, IV on-by-default, or one agreed default). C -&gt; the two reports are documented as deliberately different and our cross-case contradiction is closed by writing each report's own model down.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>item 7 of the 17-item sheet</t>
+          <t>item 6 of the 17-item sheet</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
@@ -2943,12 +2918,12 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>asked once, as Tab 2 item 1</t>
+          <t>asked once, as Tab 2 item 2</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off</t>
+          <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off [this is the grouped mapping row the source sheet used for its items 6-12; "row 2" in its text means the sheet's own item-2 row, which is carried above as Tab 3 item 2]</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
@@ -2965,123 +2940,138 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
+          <t>item 7 of the 17-item sheet</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>PO-Questions-Chris-ReportSuite-2026-08-03 (the 17-item sheet)</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>asked once, as Tab 2 item 1</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off [this is the grouped mapping row the source sheet used for its items 6-12; "row 2" in its text means the sheet's own item-2 row, which is carried above as Tab 3 item 2]</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>Named individually at the QA lead's instruction ("each named individually, not as a bundle"), because the 2026-08-04 deadline is tomorrow and a bundled question has so far produced a bundled non-answer.</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>No case change on any answer - the cases already follow his rulings (Rule 32). These only close a documentation debt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
           <t>item 13 of the 17-item sheet</t>
         </is>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>PO-Questions-Chris-ReportSuite-2026-08-03 (the 17-item sheet)</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
-        <is>
-          <t>asked once, as Tab 2 item 9</t>
-        </is>
-      </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>asked once, as Tab 2 item 8</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>PV-PERM-01 (C30325); PV-PERM-03 (C30327); PV-API-04 (C30391); IV-PERM-01 (C30603); IV-PERM-02 (C30604); TU-NAV-07 (C30398); WIP-PERM-01 (C30526); WIP-PERM-02 (C30527); PV-NAV-01 (C30322); IV-NAV-01 (C30534); TU-NAV-01 (C30392); WIP-TAB-01 (C30451)</t>
         </is>
       </c>
-      <c r="E53" s="6" t="inlineStr">
+      <c r="E54" s="6" t="inlineStr">
         <is>
           <t>NEW spec debt created by his own Q2=A ("Collapse all report access into a single Reports permission") plus the QA lead's ruling 2026-08-03, verbatim: "Yes all the reports will be gated by ONE permission FOR NOW." Verified live 2026-08-03: PV S1-R4/S1-N2, IV S1-R4 and the TU/WIP Story-1 prerequisites still name per-area permissions; only SBC S1-R2 has been corrected (2026-07-31). NOTE: the SBC change log still instructs engineering to DROP the atom, while his later chat allows hiding it inert - the later source wins (Rule 32).</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr">
+      <c r="F54" s="6" t="inlineStr">
         <is>
           <t>No decision needed - the model is settled. Groups C and D of staged-case-plan-CDE-2026-08-03.md reword these 12 cases to the single permission; the two retire-or-rescope candidates (C30327, C30391) await the QA lead's sign-off.</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="1" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
         <is>
           <t>CHANGES MADE IN CONSOLIDATION - ALL OF THEM</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>Where</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>What changed</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>Why</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="6" t="inlineStr">
-        <is>
-          <t>Tab 1 opening line</t>
-        </is>
-      </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>The original said the question is "separate from the longer sheet you already have - that one still stands". Now that the three sheets are one workbook it points at the other two tabs instead. No change of meaning.</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="inlineStr">
-        <is>
-          <t>pointer fix, forced by the consolidation</t>
-        </is>
-      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>Tab 2 opening line — the item count</t>
+          <t>Tab 1 opening line</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>"There are 10 items: 8 need you to choose something..." recomputed to 9 items / 7 decisions, because item 2 moved to Tab 1. The counts are computed from the data, never typed, so they cannot drift again.</t>
+          <t>The original said the question is "separate from the longer sheet you already have - that one still stands". Now that the three sheets are one workbook it points at the other two tabs instead. No change of meaning.</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>stale figure, caused by the de-duplication</t>
+          <t>pointer fix, forced by the consolidation</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>Tab 2 opening line — the companion pointer</t>
+          <t>Tab 2 opening line — the item count</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>"Please read it alongside the sheet dated 3 August" now reads "the last tab is its companion". Same sentence otherwise.</t>
+          <t>"There are 10 items: 8 need you to choose something..." recomputed to 9 items / 7 decisions, because item 2 moved to Tab 1. The counts are computed from the data, never typed, so they cannot drift again.</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>pointer fix, forced by the consolidation</t>
+          <t>stale figure, caused by the de-duplication</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>Tab 2 opening line — "this sheet"</t>
+          <t>Tab 2 opening line — the companion pointer</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>The two occurrences of "this sheet" read "this tab". Nothing else in the paragraph changed.</t>
+          <t>"Please read it alongside the sheet dated 3 August" now reads "the last tab is its companion". Same sentence otherwise.</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -3093,176 +3083,166 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>Tab 3, item 2 — the pointer at the end</t>
+          <t>Tab 2 opening line — "this sheet"</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>"The seven still-missing edits are listed one by one further down this sheet" now reads "...are each listed on their own further down, or on the tab before this one where the product disagrees with your answer as well" — because two of those seven (the vehicle number on Work In Progress, and the location chooser) are now asked once, on Tab 2.</t>
+          <t>The two occurrences of "this sheet" read "this tab". Nothing else in the paragraph changed.</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>pointer fix, forced by the de-duplication</t>
+          <t>pointer fix, forced by the consolidation</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>QA-only tab — the "not asked here" rows that pointed at the other sheet</t>
+          <t>Tab 3, item 2 — the pointer at the end</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>Five rows said "already question N of the 3 August sheet". They now name the tab and item number in this workbook. One row — "the 17 items of the 3 August sheet are deliberately not duplicated" — became meaningless once the sheets merged and is replaced by a row describing the consolidation itself.</t>
+          <t>"The seven still-missing edits are listed one by one further down this sheet" now reads "...are each listed on their own further down, or on the tab before this one where the product disagrees with your answer as well" — because two of those seven (the vehicle number on Work In Progress, and the location chooser) are now asked once, on Tab 2.</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>pointer fix, forced by the consolidation</t>
+          <t>pointer fix, forced by the de-duplication</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
+          <t>QA-only tab — the "not asked here" rows that pointed at the other sheet</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>Five rows said "already question N of the 3 August sheet". They now name the tab and item number in this workbook. One row — "the 17 items of the 3 August sheet are deliberately not duplicated" — became meaningless once the sheets merged and is replaced by a row describing the consolidation itself.</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>pointer fix, forced by the consolidation</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="inlineStr">
+        <is>
           <t>QA-only tab — the source-currency block</t>
         </is>
       </c>
-      <c r="B63" s="6" t="inlineStr">
+      <c r="B64" s="6" t="inlineStr">
         <is>
           <t>The six description versions were RE-CHECKED LIVE today, 2026-08-04, read straight from Confluence rather than carried over from the 3 August check. All six are unchanged (Sales By Customer 13 · Sales By Representative 15 · Parts Velocity 4 · Technician Utilization 5 · Work In Progress 6 · Inventory Value 3), so no item on any tab has been overtaken by a description edit. Dates and verdicts updated accordingly.</t>
         </is>
       </c>
-      <c r="C63" s="6" t="inlineStr">
+      <c r="C64" s="6" t="inlineStr">
         <is>
           <t>Standing Rule 31 pre-flight, done fresh for this pass</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="1" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="1" t="inlineStr">
         <is>
           <t>DECLARED WORDING CARRY-OVER (STANDING RULE 7)</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
         <is>
           <t>Word</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B67" s="3" t="inlineStr">
         <is>
           <t>Where</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr">
+      <c r="C67" s="3" t="inlineStr">
         <is>
           <t>Why it is kept rather than reworded</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="6" t="inlineStr">
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
         <is>
           <t>toggle</t>
         </is>
       </c>
-      <c r="B67" s="6" t="inlineStr">
+      <c r="B68" s="6" t="inlineStr">
         <is>
           <t>Tab 3 item 10</t>
         </is>
       </c>
-      <c r="C67" s="6" t="inlineStr">
+      <c r="C68" s="6" t="inlineStr">
         <is>
           <t>The phrase "a select-all / clear-all toggle" is carried VERBATIM from the 3 August sheet, which is wording-checked and ready to send. "Toggle" is also Chris's own vocabulary — his Inventory Value description says "it is not a user-toggled column in the column-selection control" — so it is his word, not our jargon. Rewriting a wording-checked, PO-facing line was outside the brief for this pass, so it is declared instead of silently changed.</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="1" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="1" t="inlineStr">
         <is>
           <t>SOURCE-CURRENCY BLOCK (STANDING RULE 31)</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="3" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
+      <c r="B71" s="3" t="inlineStr">
         <is>
           <t>Identifier</t>
         </is>
       </c>
-      <c r="C70" s="3" t="inlineStr">
+      <c r="C71" s="3" t="inlineStr">
         <is>
           <t>Version / last-updated</t>
         </is>
       </c>
-      <c r="D70" s="3" t="inlineStr">
+      <c r="D71" s="3" t="inlineStr">
         <is>
           <t>Checked</t>
         </is>
       </c>
-      <c r="E70" s="3" t="inlineStr">
+      <c r="E71" s="3" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="6" t="inlineStr">
-        <is>
-          <t>Sales By Customer description</t>
-        </is>
-      </c>
-      <c r="B71" s="6" t="inlineStr">
-        <is>
-          <t>Confluence page 577634305</t>
-        </is>
-      </c>
-      <c r="C71" s="6" t="inlineStr">
-        <is>
-          <t>version 13, last changed 2026-07-31</t>
-        </is>
-      </c>
-      <c r="D71" s="6" t="inlineStr">
-        <is>
-          <t>2026-08-04 (read live)</t>
-        </is>
-      </c>
-      <c r="E71" s="6" t="inlineStr">
-        <is>
-          <t>CURRENT - unchanged since the sheets were written</t>
-        </is>
-      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>Sales By Representative description</t>
+          <t>Sales By Customer description</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Confluence page 585629698</t>
+          <t>Confluence page 577634305</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>version 15, last changed 2026-07-29</t>
+          <t>version 13, last changed 2026-07-31</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
@@ -3279,17 +3259,17 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>Parts Velocity description</t>
+          <t>Sales By Representative description</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Confluence page 620888066</t>
+          <t>Confluence page 585629698</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>version 4, last changed 2026-07-29</t>
+          <t>version 15, last changed 2026-07-29</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
@@ -3306,17 +3286,17 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>Technician Utilization description</t>
+          <t>Parts Velocity description</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Confluence page 641400833</t>
+          <t>Confluence page 620888066</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>version 5, last changed 2026-07-29</t>
+          <t>version 4, last changed 2026-07-29</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
@@ -3333,17 +3313,17 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>Work In Progress description</t>
+          <t>Technician Utilization description</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>Confluence page 703660034</t>
+          <t>Confluence page 641400833</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>version 6, last changed 2026-07-29</t>
+          <t>version 5, last changed 2026-07-29</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
@@ -3360,17 +3340,17 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>Inventory Value description</t>
+          <t>Work In Progress description</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>Confluence page 720142338</t>
+          <t>Confluence page 703660034</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>version 3, last changed 2026-07-29</t>
+          <t>version 6, last changed 2026-07-29</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
@@ -3387,98 +3367,98 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>The build</t>
+          <t>Inventory Value description</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>QA branch sv8582 / project/reports-suite-bravo, app-version v3.4.1-0ed4433</t>
+          <t>Confluence page 720142338</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>v3.4.1-0ed4433</t>
+          <t>version 3, last changed 2026-07-29</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>2026-08-03 / 2026-08-04</t>
+          <t>2026-08-04 (read live)</t>
         </is>
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>PARTIAL - engineering declared the branch NOT FINAL, so every observation quoted on these tabs is PROVISIONAL and is queued for re-check in viu-2026-08-03/RECHECK-QUEUE.md (Standing Rule 49). Shortfall: the observations may change when the branch settles.</t>
+          <t>CURRENT - unchanged since the sheets were written</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>Epic SV-8582 + child stories</t>
+          <t>The build</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>Jira, project SV</t>
+          <t>QA branch sv8582 / project/reports-suite-bravo, app-version v3.4.1-0ed4433</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>currency-checked, no full re-read this pass</t>
+          <t>v3.4.1-0ed4433</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-03 / 2026-08-04</t>
         </is>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>PARTIAL - Tier-1 currency check only (Standing Rule 37); a full re-read was not authorised for this pass and is not claimed</t>
+          <t>PARTIAL - engineering declared the branch NOT FINAL, so every observation quoted on these tabs is PROVISIONAL and is queued for re-check in viu-2026-08-03/RECHECK-QUEUE.md (Standing Rule 49). Shortfall: the observations may change when the branch settles.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>Designs</t>
+          <t>Epic SV-8582 + child stories</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>none exist for the Report Suite</t>
+          <t>Jira, project SV</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>currency-checked, no full re-read this pass</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>ABSENT - spec-only project; no Figma file has ever been supplied, so no design source was consulted and none is claimed</t>
+          <t>PARTIAL - Tier-1 currency check only (Standing Rule 37); a full re-read was not authorised for this pass and is not claimed</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>Engineering tech plan</t>
+          <t>Designs</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>tech-plan-2026-07-29/</t>
+          <t>none exist for the Report Suite</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>as supplied 2026-07-29</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
@@ -3488,24 +3468,24 @@
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t>CURRENT</t>
+          <t>ABSENT - spec-only project; no Figma file has ever been supplied, so no design source was consulted and none is claimed</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>Chris Ward's answers, messages and both videos</t>
+          <t>Engineering tech plan</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>chris-answers-2026-07-28 / -07-31 / -08-01, chris-update-2026-07-29, both video transcripts</t>
+          <t>tech-plan-2026-07-29/</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>newest = the 2026-08-01-round two-question sheet</t>
+          <t>as supplied 2026-07-29</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
@@ -3515,109 +3495,114 @@
       </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>CURRENT - re-swept today; nothing newer than 2026-08-01 exists, so no question on any tab has been answered since the source sheets were written</t>
+          <t>CURRENT</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
+          <t>Chris Ward's answers, messages and both videos</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>chris-answers-2026-07-28 / -07-31 / -08-01, chris-update-2026-07-29, both video transcripts</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>newest = the 2026-08-01-round two-question sheet</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>CURRENT - re-swept today; nothing newer than 2026-08-01 exists, so no question on any tab has been answered since the source sheets were written</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
           <t>The three source sheets themselves</t>
         </is>
       </c>
-      <c r="B82" s="6" t="inlineStr">
+      <c r="B83" s="6" t="inlineStr">
         <is>
           <t>chris-location-question-2026-08-04 / chris-sheet-2026-08-04 / PO-Questions-Chris-ReportSuite-2026-08-03</t>
         </is>
       </c>
-      <c r="C82" s="6" t="inlineStr">
+      <c r="C83" s="6" t="inlineStr">
         <is>
           <t>all three READY TO SEND, none sent</t>
         </is>
       </c>
-      <c r="D82" s="6" t="inlineStr">
+      <c r="D83" s="6" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="E82" s="6" t="inlineStr">
+      <c r="E83" s="6" t="inlineStr">
         <is>
           <t>CURRENT - all three are now marked SUPERSEDED by this workbook, and are kept, not deleted</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="6" t="inlineStr">
-        <is>
-          <t>Method (Standing Rule 31, and the version-number trap it names): the six description versions were read from the LIVE Confluence page objects on 2026-08-04 - GET /wiki/api/v2/pages/&lt;id&gt;, HTTP 200 on all six - and the CONFLUENCE VERSION NUMBER was used, never the version written inside the document body. Values read: 13 (2026-07-31), 15, 4, 5, 6, 3 (all five 2026-07-29). These are the exact versions the three source sheets were built against, so nothing on any tab is stale against its description.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
+          <t>Method (Standing Rule 31, and the version-number trap it names): the six description versions were read from the LIVE Confluence page objects on 2026-08-04 - GET /wiki/api/v2/pages/&lt;id&gt;, HTTP 200 on all six - and the CONFLUENCE VERSION NUMBER was used, never the version written inside the document body. Values read: 13 (2026-07-31), 15, 4, 5, 6, 3 (all five 2026-07-29). These are the exact versions the three source sheets were built against, so nothing on any tab is stale against its description.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
           <t>Build marker: v3.4.1-0ed4433 - the branch is NOT FINAL, so every observation is PROVISIONAL (Standing Rule 49; re-check queue viu-2026-08-03/RECHECK-QUEUE.md is OPEN).</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="1" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="1" t="inlineStr">
         <is>
           <t>COMPLETENESS PROOF - EVERY SOURCE SWEPT (STANDING RULE 17)</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="3" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B88" s="3" t="inlineStr">
+      <c r="B89" s="3" t="inlineStr">
         <is>
           <t>Items found</t>
         </is>
       </c>
-      <c r="C88" s="3" t="inlineStr">
+      <c r="C89" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="D88" s="3" t="inlineStr">
+      <c r="D89" s="3" t="inlineStr">
         <is>
           <t>Swept by</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
-      <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="6" t="inlineStr">
-        <is>
-          <t>viu-2026-08-03/batch-sbc-sbr/VERDICTS.md + STAGED-CHANGES.md</t>
-        </is>
-      </c>
-      <c r="B89" s="6" t="inlineStr">
-        <is>
-          <t>3 spec-vs-build items</t>
-        </is>
-      </c>
-      <c r="C89" s="6" t="inlineStr">
-        <is>
-          <t>items 4, 5, 6 (SBC/SBR halves) and 10. The SBC nav-group question (spec says Performance, build says SALES) is NOT on this sheet - it is already question 9 of the 3 August sheet, unanswered</t>
-        </is>
-      </c>
-      <c r="D89" s="6" t="inlineStr">
-        <is>
-          <t>the 10-row sheet</t>
-        </is>
-      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>viu-2026-08-03/batch-pv-tu/VERDICTS.md + STAGED-CHANGES.md</t>
+          <t>viu-2026-08-03/batch-sbc-sbr/VERDICTS.md + STAGED-CHANGES.md</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
@@ -3627,7 +3612,7 @@
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>items 1 (PV/TU halves), 6 (PV half) and 7. Its section-C product questions map 1:1 onto items 1, 6 and 7</t>
+          <t>items 4, 5, 6 (SBC/SBR halves) and 10. The SBC nav-group question (spec says Performance, build says SALES) is NOT on this sheet - it is already question 9 of the 3 August sheet, unanswered</t>
         </is>
       </c>
       <c r="D90" s="6" t="inlineStr">
@@ -3639,17 +3624,17 @@
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>viu-2026-08-03/batch-wip-iv/VERDICTS.md + STAGED-CHANGES.md</t>
+          <t>viu-2026-08-03/batch-pv-tu/VERDICTS.md + STAGED-CHANGES.md</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>4 spec-vs-build items</t>
+          <t>3 spec-vs-build items</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>items 1 (WIP/IV halves), 2, 3 and 8. Its group C (HELD pending a Chris ruling, 6 cases) is fully represented here: C1 -&gt; item 3, C2 -&gt; item 1, C3 is a build defect not a product question</t>
+          <t>items 1 (PV/TU halves), 6 (PV half) and 7. Its section-C product questions map 1:1 onto items 1, 6 and 7</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
@@ -3661,17 +3646,17 @@
     <row r="92">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>viu-2026-08-03/LABEL-DIFF.md</t>
+          <t>viu-2026-08-03/batch-wip-iv/VERDICTS.md + STAGED-CHANGES.md</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>4 items</t>
+          <t>4 spec-vs-build items</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>A2 -&gt; item 7, A3 -&gt; item 6, A4 -&gt; item 4, A5 -&gt; item 5. A6/A7/A8/A9 are build defects or wording fixes, not product decisions - excluded with reason</t>
+          <t>items 1 (WIP/IV halves), 2, 3 and 8. Its group C (HELD pending a Chris ruling, 6 cases) is fully represented here: C1 -&gt; item 3, C2 -&gt; item 1, C3 is a build defect not a product question</t>
         </is>
       </c>
       <c r="D92" s="6" t="inlineStr">
@@ -3683,17 +3668,17 @@
     <row r="93">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>viu-2026-08-03/SURFACE-MATRIX.md</t>
+          <t>viu-2026-08-03/LABEL-DIFF.md</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>2 items</t>
+          <t>4 items</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>Matrix 2 -&gt; item 9; the 1b as-of/locations line sweep -&gt; item 8. Matrix 1a (Location column placement) is read as an implementation slip with no product question</t>
+          <t>A2 -&gt; item 7, A3 -&gt; item 6, A4 -&gt; item 4, A5 -&gt; item 5. A6/A7/A8/A9 are build defects or wording fixes, not product decisions - excluded with reason</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
@@ -3705,17 +3690,17 @@
     <row r="94">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>viu-2026-08-03/DELIBERATE-DECISIONS.md</t>
+          <t>viu-2026-08-03/SURFACE-MATRIX.md</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>4 of 35 entries name Chris Ward as the closer</t>
+          <t>2 items</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>1.4 -&gt; item 10, 2.1 -&gt; item 6, 2.4 -&gt; item 7; the fourth (logo treatment) is already question 4 of the 3 August sheet and is NOT repeated</t>
+          <t>Matrix 2 -&gt; item 9; the 1b as-of/locations line sweep -&gt; item 8. Matrix 1a (Location column placement) is read as an implementation slip with no product question</t>
         </is>
       </c>
       <c r="D94" s="6" t="inlineStr">
@@ -3727,17 +3712,17 @@
     <row r="95">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>viu-2026-08-03/RECHECK-QUEUE.md</t>
+          <t>viu-2026-08-03/DELIBERATE-DECISIONS.md</t>
         </is>
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>0 new</t>
+          <t>4 of 35 entries name Chris Ward as the closer</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>B18/B19/B34 are the same observations as items 1, 7 and 2. Every row on this sheet inherits the queue's PROVISIONAL status (Standing Rule 49)</t>
+          <t>1.4 -&gt; item 10, 2.1 -&gt; item 6, 2.4 -&gt; item 7; the fourth (logo treatment) is already question 4 of the 3 August sheet and is NOT repeated</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
@@ -3749,7 +3734,7 @@
     <row r="96">
       <c r="A96" s="6" t="inlineStr">
         <is>
-          <t>spec-watch-verification-2026-08-03/VERIFICATION.md + ADDENDUM</t>
+          <t>viu-2026-08-03/RECHECK-QUEUE.md</t>
         </is>
       </c>
       <c r="B96" s="6" t="inlineStr">
@@ -3759,7 +3744,7 @@
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>confirms the six live versions used in the source-currency block (SBC 13 / SBR 15 / PV 4 / TU 5 / WIP 6 / IV 3) and that only SBC moved since 07-31</t>
+          <t>B18/B19/B34 are the same observations as items 1, 7 and 2. Every row on this sheet inherits the queue's PROVISIONAL status (Standing Rule 49)</t>
         </is>
       </c>
       <c r="D96" s="6" t="inlineStr">
@@ -3771,17 +3756,17 @@
     <row r="97">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>The six live descriptions, re-read for this sheet</t>
+          <t>spec-watch-verification-2026-08-03/VERIFICATION.md + ADDENDUM</t>
         </is>
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>10 verbatim quotes extracted</t>
+          <t>0 new</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>every reader-facing quote on this sheet was pulled from the live capture or the version-matched mirror, not from a summary (Standing Rule 15)</t>
+          <t>confirms the six live versions used in the source-currency block (SBC 13 / SBR 15 / PV 4 / TU 5 / WIP 6 / IV 3) and that only SBC moved since 07-31</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
@@ -3793,17 +3778,17 @@
     <row r="98">
       <c r="A98" s="6" t="inlineStr">
         <is>
-          <t>PO-Questions-Chris-ReportSuite-2026-08-03.md (17 items, unanswered)</t>
+          <t>The six live descriptions, re-read for this sheet</t>
         </is>
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>0 duplicated</t>
+          <t>10 verbatim quotes extracted</t>
         </is>
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>checked item by item - nothing on this sheet repeats it. Its 17 items are description-text asks; this sheet is spec-versus-build behaviour. The overlap is only item 9 here vs its item 13, and ours adds the live both-ways proof it lacked</t>
+          <t>every reader-facing quote on this sheet was pulled from the live capture or the version-matched mirror, not from a summary (Standing Rule 15)</t>
         </is>
       </c>
       <c r="D98" s="6" t="inlineStr">
@@ -3815,17 +3800,17 @@
     <row r="99">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>chris-answers-2026-07-28 / -07-31 / -08-01, chris-update-2026-07-29, both videos</t>
+          <t>PO-Questions-Chris-ReportSuite-2026-08-03.md (17 items, unanswered)</t>
         </is>
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>8 candidates WITHDRAWN</t>
+          <t>0 duplicated</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>see the withdrawn appendix - every one quoted</t>
+          <t>checked item by item - nothing on this sheet repeats it. Its 17 items are description-text asks; this sheet is spec-versus-build behaviour. The overlap is only item 9 here vs its item 13, and ours adds the live both-ways proof it lacked</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
@@ -3837,17 +3822,17 @@
     <row r="100">
       <c r="A100" s="6" t="inlineStr">
         <is>
-          <t>coverage-rederivation-2026-07-31/DELIBERATE-DECISIONS.md + COVERAGE-REDERIVATION.md</t>
+          <t>chris-answers-2026-07-28 / -07-31 / -08-01, chris-update-2026-07-29, both videos</t>
         </is>
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>0 new</t>
+          <t>8 candidates WITHDRAWN</t>
         </is>
       </c>
       <c r="C100" s="6" t="inlineStr">
         <is>
-          <t>its open bucket is fully covered by the 3 August sheet; nothing there is a spec-vs-build item</t>
+          <t>see the withdrawn appendix - every one quoted</t>
         </is>
       </c>
       <c r="D100" s="6" t="inlineStr">
@@ -3859,7 +3844,7 @@
     <row r="101">
       <c r="A101" s="6" t="inlineStr">
         <is>
-          <t>OUTSTANDING-ITEMS-REGISTER.md (Report Suite rows)</t>
+          <t>coverage-rederivation-2026-07-31/DELIBERATE-DECISIONS.md + COVERAGE-REDERIVATION.md</t>
         </is>
       </c>
       <c r="B101" s="6" t="inlineStr">
@@ -3869,7 +3854,7 @@
       </c>
       <c r="C101" s="6" t="inlineStr">
         <is>
-          <t>its Chris-facing rows are the 3 August sheet itself and the spec-watch deadline; the QA-branch row is the QA lead's, not Chris's</t>
+          <t>its open bucket is fully covered by the 3 August sheet; nothing there is a spec-vs-build item</t>
         </is>
       </c>
       <c r="D101" s="6" t="inlineStr">
@@ -3881,39 +3866,39 @@
     <row r="102">
       <c r="A102" s="6" t="inlineStr">
         <is>
-          <t>PO-Questions-Chris-ReportSuite-2026-07-31.md (5 questions)</t>
+          <t>OUTSTANDING-ITEMS-REGISTER.md (Report Suite rows)</t>
         </is>
       </c>
       <c r="B102" s="6" t="inlineStr">
         <is>
-          <t>4 open</t>
+          <t>0 new</t>
         </is>
       </c>
       <c r="C102" s="6" t="inlineStr">
         <is>
-          <t>Q5 is ANSWERED (=A) on the separate permissions sheet; Q1-Q4 carried forward VERBATIM</t>
+          <t>its Chris-facing rows are the 3 August sheet itself and the spec-watch deadline; the QA-branch row is the QA lead's, not Chris's</t>
         </is>
       </c>
       <c r="D102" s="6" t="inlineStr">
         <is>
-          <t>the 17-item sheet</t>
+          <t>the 10-row sheet</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>PO-Questions-Chris-ReportSuite-2026-07-27.md (3 questions)</t>
+          <t>PO-Questions-Chris-ReportSuite-2026-07-31.md (5 questions)</t>
         </is>
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>0 open</t>
+          <t>4 open</t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
         <is>
-          <t>Q1 answered 2026-07-28 ("B."), Q2 superseded by the one-permission ruling, Q3 answered by the 2026-07-30 Loom</t>
+          <t>Q5 is ANSWERED (=A) on the separate permissions sheet; Q1-Q4 carried forward VERBATIM</t>
         </is>
       </c>
       <c r="D103" s="6" t="inlineStr">
@@ -3925,7 +3910,7 @@
     <row r="104">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>PO-Questions-Chris-ReportSuite-TechPlan_2026-07-30.md (5 questions)</t>
+          <t>PO-Questions-Chris-ReportSuite-2026-07-27.md (3 questions)</t>
         </is>
       </c>
       <c r="B104" s="6" t="inlineStr">
@@ -3935,7 +3920,7 @@
       </c>
       <c r="C104" s="6" t="inlineStr">
         <is>
-          <t>all five answered = A on 2026-07-31; 70 cases updated + 7 added and pushed</t>
+          <t>Q1 answered 2026-07-28 ("B."), Q2 superseded by the one-permission ruling, Q3 answered by the 2026-07-30 Loom</t>
         </is>
       </c>
       <c r="D104" s="6" t="inlineStr">
@@ -3947,17 +3932,17 @@
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>SPEC-WATCH-2026-07-28.md (12 items, deadline 2026-08-04)</t>
+          <t>PO-Questions-Chris-ReportSuite-TechPlan_2026-07-30.md (5 questions)</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>7 open</t>
+          <t>0 open</t>
         </is>
       </c>
       <c r="C105" s="6" t="inlineStr">
         <is>
-          <t>items 1b, 4, 6, 8, 9, 10, 11 - each now asked INDIVIDUALLY as items 6-12</t>
+          <t>all five answered = A on 2026-07-31; 70 cases updated + 7 added and pushed</t>
         </is>
       </c>
       <c r="D105" s="6" t="inlineStr">
@@ -3969,17 +3954,17 @@
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>What-We-Need-From-Chris-Ward-2026-07-31.md (12 items)</t>
+          <t>SPEC-WATCH-2026-07-28.md (12 items, deadline 2026-08-04)</t>
         </is>
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>11 open</t>
+          <t>7 open</t>
         </is>
       </c>
       <c r="C106" s="6" t="inlineStr">
         <is>
-          <t>item 4 (permission granularity) is now closed; the rest dedupe into this sheet</t>
+          <t>items 1b, 4, 6, 8, 9, 10, 11 - each now asked INDIVIDUALLY as items 6-12</t>
         </is>
       </c>
       <c r="D106" s="6" t="inlineStr">
@@ -3991,17 +3976,17 @@
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>coverage-rederivation-2026-07-31/DELIBERATE-DECISIONS.md (D1-D7 open bucket)</t>
+          <t>What-We-Need-From-Chris-Ward-2026-07-31.md (12 items)</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>6 open</t>
+          <t>11 open</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr">
         <is>
-          <t>D5 closed by the one-permission ruling; D1/D2/D3/D4/D6/D7 all dedupe into this sheet</t>
+          <t>item 4 (permission granularity) is now closed; the rest dedupe into this sheet</t>
         </is>
       </c>
       <c r="D107" s="6" t="inlineStr">
@@ -4013,17 +3998,17 @@
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>OUTSTANDING-ITEMS-REGISTER.md (Report Suite rows)</t>
+          <t>coverage-rederivation-2026-07-31/DELIBERATE-DECISIONS.md (D1-D7 open bucket)</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>0 new</t>
+          <t>6 open</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
         <is>
-          <t>its Chris-facing rows are the QA branch (not Chris), SV-8780 (out of scope by ruling) and the scope question (now answered)</t>
+          <t>D5 closed by the one-permission ruling; D1/D2/D3/D4/D6/D7 all dedupe into this sheet</t>
         </is>
       </c>
       <c r="D108" s="6" t="inlineStr">
@@ -4035,17 +4020,17 @@
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>The six LIVE Confluence specs, re-checked 2026-08-03</t>
+          <t>OUTSTANDING-ITEMS-REGISTER.md (Report Suite rows)</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>2 new</t>
+          <t>0 new</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
         <is>
-          <t>SBC lastModified Jul 31; SBR/PV/TU/WIP/IV all still Jul 29. NEW: the five per-area permission descriptions (item 13); and the SBC change log still says DROP the atom while his chat says hide it (folded into item 13's note)</t>
+          <t>its Chris-facing rows are the QA branch (not Chris), SV-8780 (out of scope by ruling) and the scope question (now answered)</t>
         </is>
       </c>
       <c r="D109" s="6" t="inlineStr">
@@ -4057,17 +4042,17 @@
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>Chris's 2026-08-01-round chat message + the filled 2-question sheet</t>
+          <t>The six LIVE Confluence specs, re-checked 2026-08-03</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>1 new</t>
+          <t>2 new</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
-          <t>"which SBC features were dropped" (item 5). His two answers themselves are ingested, not re-asked</t>
+          <t>SBC lastModified Jul 31; SBR/PV/TU/WIP/IV all still Jul 29. NEW: the five per-area permission descriptions (item 13); and the SBC change log still says DROP the atom while his chat says hide it (folded into item 13's note)</t>
         </is>
       </c>
       <c r="D110" s="6" t="inlineStr">
@@ -4079,7 +4064,7 @@
     <row r="111">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>Chris's 2026-07-29 group message</t>
+          <t>Chris's 2026-08-01-round chat message + the filled 2-question sheet</t>
         </is>
       </c>
       <c r="B111" s="6" t="inlineStr">
@@ -4089,7 +4074,7 @@
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>the "be careful with the acronym VIN" caution is his own point and is not written into any spec (item 16)</t>
+          <t>"which SBC features were dropped" (item 5). His two answers themselves are ingested, not re-asked</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
@@ -4101,17 +4086,17 @@
     <row r="112">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>Both walkthrough videos (2026-07-30 Loom + the earlier PRD companion)</t>
+          <t>Chris's 2026-07-29 group message</t>
         </is>
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>0 new</t>
+          <t>1 new</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
         <is>
-          <t>every delta already promoted or on SPEC-WATCH; nothing unaddressed</t>
+          <t>the "be careful with the acronym VIN" caution is his own point and is not written into any spec (item 16)</t>
         </is>
       </c>
       <c r="D112" s="6" t="inlineStr">
@@ -4123,7 +4108,7 @@
     <row r="113">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>coverage-rederivation-2026-07-31/COVERAGE-REDERIVATION.md (spec-silent / spec-inconsistent flags)</t>
+          <t>Both walkthrough videos (2026-07-30 Loom + the earlier PRD companion)</t>
         </is>
       </c>
       <c r="B113" s="6" t="inlineStr">
@@ -4133,7 +4118,7 @@
       </c>
       <c r="C113" s="6" t="inlineStr">
         <is>
-          <t>the spec-silent flag is the Summary-download position = item 3; the spec-inconsistent flags are items 1 and 4</t>
+          <t>every delta already promoted or on SPEC-WATCH; nothing unaddressed</t>
         </is>
       </c>
       <c r="D113" s="6" t="inlineStr">
@@ -4145,7 +4130,7 @@
     <row r="114">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>PROJECT-STATE.md</t>
+          <t>coverage-rederivation-2026-07-31/COVERAGE-REDERIVATION.md (spec-silent / spec-inconsistent flags)</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
@@ -4155,7 +4140,7 @@
       </c>
       <c r="C114" s="6" t="inlineStr">
         <is>
-          <t>no Chris-facing ask not already listed above</t>
+          <t>the spec-silent flag is the Summary-download position = item 3; the spec-inconsistent flags are items 1 and 4</t>
         </is>
       </c>
       <c r="D114" s="6" t="inlineStr">
@@ -4167,29 +4152,29 @@
     <row r="115">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>The six LIVE Confluence descriptions, re-read for THIS workbook 2026-08-04</t>
+          <t>PROJECT-STATE.md</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>**0 new**</t>
+          <t>0 new</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
         <is>
-          <t>All six still at the versions the source sheets used (13 / 15 / 4 / 5 / 6 / 3), read live over the page API, HTTP 200 on all six. No item has been overtaken by a description edit, so nothing needed withdrawing on that ground.</t>
+          <t>no Chris-facing ask not already listed above</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>this consolidation</t>
+          <t>the 17-item sheet</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>Chris Ward's answers, messages and both video transcripts, re-swept 2026-08-04</t>
+          <t>The six LIVE Confluence descriptions, re-read for THIS workbook 2026-08-04</t>
         </is>
       </c>
       <c r="B116" s="6" t="inlineStr">
@@ -4199,7 +4184,7 @@
       </c>
       <c r="C116" s="6" t="inlineStr">
         <is>
-          <t>Newest authoritative Chris source is still 2026-08-01, which both source sheets already accounted for. Nothing has been answered since they were written, so 0 further candidates were withdrawn by this pass; the 12 rows above are the de-duplicated union of what the two sheets had already withdrawn.</t>
+          <t>All six still at the versions the source sheets used (13 / 15 / 4 / 5 / 6 / 3), read live over the page API, HTTP 200 on all six. No item has been overtaken by a description edit, so nothing needed withdrawing on that ground.</t>
         </is>
       </c>
       <c r="D116" s="6" t="inlineStr">
@@ -4211,17 +4196,17 @@
     <row r="117">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>The three source sheets, compared item by item for overlap</t>
+          <t>Chris Ward's answers, messages and both video transcripts, re-swept 2026-08-04</t>
         </is>
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>**4 overlaps found**</t>
+          <t>**0 new**</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr">
         <is>
-          <t>1 the two sheets had already spotted (the permission write-down) and 3 this pass found: the Location-column model asked twice, and two write-down tick-boxes whose ask is already inside a spec-versus-build item's options. All four removed; see the de-duplication log. 28 reader-facing items in, 24 out.</t>
+          <t>Newest authoritative Chris source is still 2026-08-01, which both source sheets already accounted for. Nothing has been answered since they were written, so 0 further candidates were withdrawn by this pass; the 12 rows above are the de-duplicated union of what the two sheets had already withdrawn.</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr">
@@ -4233,79 +4218,84 @@
     <row r="118">
       <c r="A118" s="6" t="inlineStr">
         <is>
+          <t>The three source sheets, compared item by item for overlap</t>
+        </is>
+      </c>
+      <c r="B118" s="6" t="inlineStr">
+        <is>
+          <t>**4 overlaps found**</t>
+        </is>
+      </c>
+      <c r="C118" s="6" t="inlineStr">
+        <is>
+          <t>1 the two sheets had already spotted (the permission write-down) and 3 this pass found: the Location-column model asked twice, and two write-down tick-boxes whose ask is already inside a spec-versus-build item's options. All four removed; see the de-duplication log. 28 reader-facing items in, 24 out.</t>
+        </is>
+      </c>
+      <c r="D118" s="6" t="inlineStr">
+        <is>
+          <t>this consolidation</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="6" t="inlineStr">
+        <is>
           <t>build/OUTSTANDING-ITEMS-REGISTER.md (Report Suite send-list row)</t>
         </is>
       </c>
-      <c r="B118" s="6" t="inlineStr">
+      <c r="B119" s="6" t="inlineStr">
         <is>
           <t>**0 new**</t>
         </is>
       </c>
-      <c r="C118" s="6" t="inlineStr">
+      <c r="C119" s="6" t="inlineStr">
         <is>
           <t>Its Chris-facing row previously listed the three sheets; it now points at this workbook. No new ask surfaced.</t>
         </is>
       </c>
-      <c r="D118" s="6" t="inlineStr">
+      <c r="D119" s="6" t="inlineStr">
         <is>
           <t>this consolidation</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" s="1" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="1" t="inlineStr">
         <is>
           <t>WITHDRAWN - ALREADY ANSWERED, NOT ASKED (12 candidates; 0 added by this pass)</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" s="3" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
         <is>
           <t>Candidate question</t>
         </is>
       </c>
-      <c r="B121" s="3" t="inlineStr">
+      <c r="B122" s="3" t="inlineStr">
         <is>
           <t>Already answered by</t>
         </is>
       </c>
-      <c r="C121" s="3" t="inlineStr">
+      <c r="C122" s="3" t="inlineStr">
         <is>
           <t>Withdrawn on</t>
         </is>
       </c>
-      <c r="D121" t="inlineStr"/>
-      <c r="E121" t="inlineStr"/>
-      <c r="F121" t="inlineStr"/>
-      <c r="G121" t="inlineStr"/>
-    </row>
-    <row r="122">
-      <c r="A122" s="6" t="inlineStr">
-        <is>
-          <t>Should the location chooser be hidden for a one-location person?</t>
-        </is>
-      </c>
-      <c r="B122" s="6" t="inlineStr">
-        <is>
-          <t>ANSWERED 2026-07-31 Q1=A, verbatim "A -- classic spec drift". NOT re-asked. Item 1 asks a genuinely NEW question that could not exist before 3 August: the build disagrees with his ruling, so he must choose whether the product changes or the ruling does. The reader-facing text states his ruling rather than asking for it again.</t>
-        </is>
-      </c>
-      <c r="C122" s="6" t="inlineStr">
-        <is>
-          <t>both sheets</t>
-        </is>
-      </c>
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
         <is>
-          <t>Should the six reports be gated by their own dedicated permission?</t>
+          <t>Should the location chooser be hidden for a one-location person?</t>
         </is>
       </c>
       <c r="B123" s="6" t="inlineStr">
         <is>
-          <t>ANSWERED THREE TIMES: 2026-07-28 ("these should be gated by normal reports access"), 2026-07-31 Q4=A ("the intention is to not hide these from normal reports access. These were specced before CRP was built :)"), and the separate permissions sheet Q1=A. Plus the QA lead 2026-08-03: "Yes all the reports will be gated by ONE permission FOR NOW." Item 9 asks ONLY for the four spec edits and says so in its own text.</t>
+          <t>ANSWERED 2026-07-31 Q1=A, verbatim "A -- classic spec drift". NOT re-asked. Item 1 asks a genuinely NEW question that could not exist before 3 August: the build disagrees with his ruling, so he must choose whether the product changes or the ruling does. The reader-facing text states his ruling rather than asking for it again.</t>
         </is>
       </c>
       <c r="C123" s="6" t="inlineStr">
@@ -4317,12 +4307,12 @@
     <row r="124">
       <c r="A124" s="6" t="inlineStr">
         <is>
-          <t>Does the 10,000-row download limit apply to Parts Velocity, Technician Utilization and Work In Progress?</t>
+          <t>Should the six reports be gated by their own dedicated permission?</t>
         </is>
       </c>
       <c r="B124" s="6" t="inlineStr">
         <is>
-          <t>ANSWERED 2026-07-31 Q3=A, verbatim "A - this was not well thought out by me (the specs were written at different times)". Suite-wide. The three cases exist and are pushed. Only his spec edit remains, and that is already item 15 of the 3 August sheet.</t>
+          <t>ANSWERED THREE TIMES: 2026-07-28 ("these should be gated by normal reports access"), 2026-07-31 Q4=A ("the intention is to not hide these from normal reports access. These were specced before CRP was built :)"), and the separate permissions sheet Q1=A. Plus the QA lead 2026-08-03: "Yes all the reports will be gated by ONE permission FOR NOW." Item 9 asks ONLY for the four spec edits and says so in its own text.</t>
         </is>
       </c>
       <c r="C124" s="6" t="inlineStr">
@@ -4334,12 +4324,12 @@
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>Which of the two "too large to export" messages is correct?</t>
+          <t>Does the 10,000-row download limit apply to Parts Velocity, Technician Utilization and Work In Progress?</t>
         </is>
       </c>
       <c r="B125" s="6" t="inlineStr">
         <is>
-          <t>ANSWERED 2026-07-31 Q2=A, verbatim "A - great catch". One suite-wide string, and the build returns it verbatim (confirmed live 2026-08-03 on the SBC guard). Nothing left to ask.</t>
+          <t>ANSWERED 2026-07-31 Q3=A, verbatim "A - this was not well thought out by me (the specs were written at different times)". Suite-wide. The three cases exist and are pushed. Only his spec edit remains, and that is already item 15 of the 3 August sheet.</t>
         </is>
       </c>
       <c r="C125" s="6" t="inlineStr">
@@ -4351,29 +4341,29 @@
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>Should the asset identifier be the VIN chain rather than the serial number?</t>
+          <t>Which of the two "too large to export" messages is correct?</t>
         </is>
       </c>
       <c r="B126" s="6" t="inlineStr">
         <is>
-          <t>ANSWERED 2026-07-29, verbatim "A is the correct answer", with the durable instruction to apply it everywhere. Item 3 does NOT re-ask it - it reports that the build did not implement it and asks which side now moves. His own VIN/serial caution is quoted inside item 3 rather than raised as its own question, because it is his point, not ours.</t>
+          <t>ANSWERED 2026-07-31 Q2=A, verbatim "A - great catch". One suite-wide string, and the build returns it verbatim (confirmed live 2026-08-03 on the SBC guard). Nothing left to ask.</t>
         </is>
       </c>
       <c r="C126" s="6" t="inlineStr">
         <is>
-          <t>the 10-row sheet</t>
+          <t>both sheets</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="6" t="inlineStr">
         <is>
-          <t>Should "Rep" be spelled out as "Representative"?</t>
+          <t>Should the asset identifier be the VIN chain rather than the serial number?</t>
         </is>
       </c>
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>ANSWERED 2026-07-31 Q5=A, verbatim "Rep is too much slang, let's do representative everywhere". Item 4 accepts that ruling and asks only about the THIRD spelling the build produced, which did not exist as a fact until 3 August.</t>
+          <t>ANSWERED 2026-07-29, verbatim "A is the correct answer", with the durable instruction to apply it everywhere. Item 3 does NOT re-ask it - it reports that the build did not implement it and asks which side now moves. His own VIN/serial caution is quoted inside item 3 rather than raised as its own question, because it is his point, not ours.</t>
         </is>
       </c>
       <c r="C127" s="6" t="inlineStr">
@@ -4385,63 +4375,63 @@
     <row r="128">
       <c r="A128" s="6" t="inlineStr">
         <is>
-          <t>Does Escape close the "deactivate a representative" pop-up?</t>
+          <t>Should "Rep" be spelled out as "Representative"?</t>
         </is>
       </c>
       <c r="B128" s="6" t="inlineStr">
         <is>
-          <t>ANSWERED 2026-07-28, verbatim "B." - Escape must NOT dismiss it. Our case follows it; only his spec edit remains and that is item 14 of the 3 August sheet.</t>
+          <t>ANSWERED 2026-07-31 Q5=A, verbatim "Rep is too much slang, let's do representative everywhere". Item 4 accepts that ruling and asks only about the THIRD spelling the build produced, which did not exist as a fact until 3 August.</t>
         </is>
       </c>
       <c r="C128" s="6" t="inlineStr">
         <is>
-          <t>both sheets</t>
+          <t>the 10-row sheet</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>Should "All Time" be offered in the date chooser?</t>
+          <t>Does Escape close the "deactivate a representative" pop-up?</t>
         </is>
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
-          <t>ANSWERED and already implemented - he removed it (SBC 2026-07-16 change log; WIP 2026-07-21 change log, recorded as "a Chris product/UX decision"). Live check 2026-08-03: not offered anywhere. Item 6 confirms its absence as a MATCH and asks only about the nine-versus-eleven list.</t>
+          <t>ANSWERED 2026-07-28, verbatim "B." - Escape must NOT dismiss it. Our case follows it; only his spec edit remains and that is item 14 of the 3 August sheet.</t>
         </is>
       </c>
       <c r="C129" s="6" t="inlineStr">
         <is>
-          <t>the 10-row sheet</t>
+          <t>both sheets</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="6" t="inlineStr">
         <is>
-          <t>How far does "one single Reports permission" reach - do the six reports just read one permission, or are the per-area permissions merged/removed in Custom Roles?</t>
+          <t>Should "All Time" be offered in the date chooser?</t>
         </is>
       </c>
       <c r="B130" s="6" t="inlineStr">
         <is>
-          <t>ANSWERED - and this was going to be the headline question of this sheet. Chris's Q2 = A ("Collapse all report access into a single Reports permission") plus the QA LEAD's ruling 2026-08-03, verbatim: "Yes all the reports will be gated by ONE permission FOR NOW." Rule 33 - the QA lead's ruling, consistent with the PO's answer. WITHDRAWN so we do not ask a settled question. "FOR NOW" is recorded on every affected case.</t>
+          <t>ANSWERED and already implemented - he removed it (SBC 2026-07-16 change log; WIP 2026-07-21 change log, recorded as "a Chris product/UX decision"). Live check 2026-08-03: not offered anywhere. Item 6 confirms its absence as a MATCH and asks only about the nine-versus-eleven list.</t>
         </is>
       </c>
       <c r="C130" s="6" t="inlineStr">
         <is>
-          <t>the 17-item sheet</t>
+          <t>the 10-row sheet</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="6" t="inlineStr">
         <is>
-          <t>Are there any pictures or videos to check the reports against? (Question 3 of the 27 July sheet)</t>
+          <t>How far does "one single Reports permission" reach - do the six reports just read one permission, or are the per-area permissions merged/removed in Custom Roles?</t>
         </is>
       </c>
       <c r="B131" s="6" t="inlineStr">
         <is>
-          <t>ANSWERED by delivery, not by words - he produced the walkthrough Loom on 2026-07-30. It was ingested and ruled AUTHORITATIVE, and drove 3 firm deltas plus the SPEC-WATCH list. Designs remain absent, which is a separate, already-recorded fact.</t>
+          <t>ANSWERED - and this was going to be the headline question of this sheet. Chris's Q2 = A ("Collapse all report access into a single Reports permission") plus the QA LEAD's ruling 2026-08-03, verbatim: "Yes all the reports will be gated by ONE permission FOR NOW." Rule 33 - the QA lead's ruling, consistent with the PO's answer. WITHDRAWN so we do not ask a settled question. "FOR NOW" is recorded on every affected case.</t>
         </is>
       </c>
       <c r="C131" s="6" t="inlineStr">
@@ -4453,12 +4443,12 @@
     <row r="132">
       <c r="A132" s="6" t="inlineStr">
         <is>
-          <t>Does the short heading "Rep is active?" also become "Representative"?</t>
+          <t>Are there any pictures or videos to check the reports against? (Question 3 of the 27 July sheet)</t>
         </is>
       </c>
       <c r="B132" s="6" t="inlineStr">
         <is>
-          <t>ANSWERED by his 2026-07-31 Q5 = A, verbatim "slang, let's do representative everywhere" - the scope explicitly reaches the export column headers. Affects SBR-ASGN-02 (C30293).</t>
+          <t>ANSWERED by delivery, not by words - he produced the walkthrough Loom on 2026-07-30. It was ingested and ruled AUTHORITATIVE, and drove 3 firm deltas plus the SPEC-WATCH list. Designs remain absent, which is a separate, already-recorded fact.</t>
         </is>
       </c>
       <c r="C132" s="6" t="inlineStr">
@@ -4470,91 +4460,91 @@
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
         <is>
+          <t>Does the short heading "Rep is active?" also become "Representative"?</t>
+        </is>
+      </c>
+      <c r="B133" s="6" t="inlineStr">
+        <is>
+          <t>ANSWERED by his 2026-07-31 Q5 = A, verbatim "slang, let's do representative everywhere" - the scope explicitly reaches the export column headers. Affects SBR-ASGN-02 (C30293).</t>
+        </is>
+      </c>
+      <c r="C133" s="6" t="inlineStr">
+        <is>
+          <t>the 17-item sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="6" t="inlineStr">
+        <is>
           <t>What is the exact renamed "Sales Rep Assignments" file name?</t>
         </is>
       </c>
-      <c r="B133" s="6" t="inlineStr">
+      <c r="B134" s="6" t="inlineStr">
         <is>
           <t>ANSWERED by the same Q5 = A - the file name is explicitly in scope of "representative everywhere". SBR-ASGN-02 (C30293) hedges the exact final string for live confirmation, which is the correct treatment; no product question remains.</t>
         </is>
       </c>
-      <c r="C133" s="6" t="inlineStr">
+      <c r="C134" s="6" t="inlineStr">
         <is>
           <t>the 17-item sheet</t>
         </is>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" s="1" t="inlineStr">
+    <row r="136">
+      <c r="A136" s="1" t="inlineStr">
         <is>
           <t>NOT ASKED HERE (QA REFERENCE)</t>
         </is>
       </c>
     </row>
-    <row r="136">
-      <c r="A136" s="3" t="inlineStr">
+    <row r="137">
+      <c r="A137" s="3" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B136" s="3" t="inlineStr">
+      <c r="B137" s="3" t="inlineStr">
         <is>
           <t>Why it is not on any tab</t>
         </is>
       </c>
-      <c r="C136" s="3" t="inlineStr">
+      <c r="C137" s="3" t="inlineStr">
         <is>
           <t>From</t>
         </is>
       </c>
-      <c r="D136" t="inlineStr"/>
-      <c r="E136" t="inlineStr"/>
-      <c r="F136" t="inlineStr"/>
-      <c r="G136" t="inlineStr"/>
-    </row>
-    <row r="137">
-      <c r="A137" s="6" t="inlineStr">
-        <is>
-          <t>Sending the three sheets separately.</t>
-        </is>
-      </c>
-      <c r="B137" s="6" t="inlineStr">
-        <is>
-          <t>REPLACED BY THIS WORKBOOK. The 10-row sheet carried a row explaining that the 17 items of the 3 August sheet were deliberately NOT duplicated; that row is meaningless now the three are one workbook. What replaces it: the three sheets are consolidated, most-urgent tab first, and FOUR overlapping items were removed so nothing is asked twice - see the de-duplication log above. The source sheets are marked SUPERSEDED and kept, not deleted.</t>
-        </is>
-      </c>
-      <c r="C137" s="6" t="inlineStr">
-        <is>
-          <t>this consolidation</t>
-        </is>
-      </c>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
         <is>
-          <t>Where the location column sits in the shorter Summary downloads (spec-silent).</t>
+          <t>Sending the three sheets separately.</t>
         </is>
       </c>
       <c r="B138" s="6" t="inlineStr">
         <is>
-          <t>Asked once, as item 3 of the third tab.</t>
+          <t>REPLACED BY THIS WORKBOOK. The 10-row sheet carried a row explaining that the 17 items of the 3 August sheet were deliberately NOT duplicated; that row is meaningless now the three are one workbook. What replaces it: the three sheets are consolidated, most-urgent tab first, and FOUR overlapping items were removed so nothing is asked twice - see the de-duplication log above. The source sheets are marked SUPERSEDED and kept, not deleted.</t>
         </is>
       </c>
       <c r="C138" s="6" t="inlineStr">
         <is>
-          <t>the 10-row sheet</t>
+          <t>this consolidation</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>"The same logo treatment" - three descriptions describe three different rules.</t>
+          <t>Where the location column sits in the shorter Summary downloads (spec-silent).</t>
         </is>
       </c>
       <c r="B139" s="6" t="inlineStr">
         <is>
-          <t>Asked once, as item 4 of the third tab.</t>
+          <t>Asked once, as item 3 of the third tab.</t>
         </is>
       </c>
       <c r="C139" s="6" t="inlineStr">
@@ -4566,12 +4556,12 @@
     <row r="140">
       <c r="A140" s="6" t="inlineStr">
         <is>
-          <t>Which Sales By Customer features were dropped.</t>
+          <t>"The same logo treatment" - three descriptions describe three different rules.</t>
         </is>
       </c>
       <c r="B140" s="6" t="inlineStr">
         <is>
-          <t>Asked once, as item 5 of the third tab.</t>
+          <t>Asked once, as item 4 of the third tab.</t>
         </is>
       </c>
       <c r="C140" s="6" t="inlineStr">
@@ -4583,12 +4573,12 @@
     <row r="141">
       <c r="A141" s="6" t="inlineStr">
         <is>
-          <t>The Sales By Customer navigation group (description says Performance, build shows SALES).</t>
+          <t>Which Sales By Customer features were dropped.</t>
         </is>
       </c>
       <c r="B141" s="6" t="inlineStr">
         <is>
-          <t>Asked once, as items 6 and 7 of the third tab. Not repeated, although the build observation is new - it is recorded in batch-sbc-sbr/STAGED-CHANGES.md for whenever he answers.</t>
+          <t>Asked once, as item 5 of the third tab.</t>
         </is>
       </c>
       <c r="C141" s="6" t="inlineStr">
@@ -4600,12 +4590,12 @@
     <row r="142">
       <c r="A142" s="6" t="inlineStr">
         <is>
-          <t>Two printable downloads fail with a server error at full size (Parts Velocity, Inventory Value).</t>
+          <t>The Sales By Customer navigation group (description says Performance, build shows SALES).</t>
         </is>
       </c>
       <c r="B142" s="6" t="inlineStr">
         <is>
-          <t>A DEFECT, not a product decision - Standing Rule 7 forbids putting bugs in front of the PO. It is a dev ticket; the friendly over-size guard exists on the spreadsheet path and the printable path fails instead of using it. Request ids captured in batch-wip-iv/evidence/api/.</t>
+          <t>Asked once, as items 6 and 7 of the third tab. Not repeated, although the build observation is new - it is recorded in batch-sbc-sbr/STAGED-CHANGES.md for whenever he answers.</t>
         </is>
       </c>
       <c r="C142" s="6" t="inlineStr">
@@ -4617,12 +4607,12 @@
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
         <is>
-          <t>The location column's on-screen POSITION on Parts Velocity and Technician Utilization (sixth/second, not leftmost).</t>
+          <t>Two printable downloads fail with a server error at full size (Parts Velocity, Inventory Value).</t>
         </is>
       </c>
       <c r="B143" s="6" t="inlineStr">
         <is>
-          <t>Read as an implementation slip, not a product decision - no source asks for anything other than leftmost, so there is nothing for him to choose. Dev ticket.</t>
+          <t>A DEFECT, not a product decision - Standing Rule 7 forbids putting bugs in front of the PO. It is a dev ticket; the friendly over-size guard exists on the spreadsheet path and the printable path fails instead of using it. Request ids captured in batch-wip-iv/evidence/api/.</t>
         </is>
       </c>
       <c r="C143" s="6" t="inlineStr">
@@ -4634,12 +4624,12 @@
     <row r="144">
       <c r="A144" s="6" t="inlineStr">
         <is>
-          <t>The Work In Progress Estimates figure showing zero, and "Inv. Hrs" being shown but not downloadable.</t>
+          <t>The location column's on-screen POSITION on Parts Velocity and Technician Utilization (sixth/second, not leftmost).</t>
         </is>
       </c>
       <c r="B144" s="6" t="inlineStr">
         <is>
-          <t>Defects. Dev tickets, not PO questions.</t>
+          <t>Read as an implementation slip, not a product decision - no source asks for anything other than leftmost, so there is nothing for him to choose. Dev ticket.</t>
         </is>
       </c>
       <c r="C144" s="6" t="inlineStr">
@@ -4651,12 +4641,12 @@
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>The QA branch being non-final, and fresh sign-in credentials.</t>
+          <t>The Work In Progress Estimates figure showing zero, and "Inv. Hrs" being shown but not downloadable.</t>
         </is>
       </c>
       <c r="B145" s="6" t="inlineStr">
         <is>
-          <t>Not Chris's to give - the QA lead's / engineering's. Every observation on this sheet is PROVISIONAL until the branch is declared final (Standing Rule 49); the re-check queue is OPEN.</t>
+          <t>Defects. Dev tickets, not PO questions.</t>
         </is>
       </c>
       <c r="C145" s="6" t="inlineStr">
@@ -4668,29 +4658,29 @@
     <row r="146">
       <c r="A146" s="6" t="inlineStr">
         <is>
-          <t>The 5 automated cases in our Report Suite folder authored by Vladimir Tomovic (C38919-C38923).</t>
+          <t>The QA branch being non-final, and fresh sign-in credentials.</t>
         </is>
       </c>
       <c r="B146" s="6" t="inlineStr">
         <is>
-          <t>Not a Chris question, and by the QA lead's ruling 2026-07-31 we do not message Vladimir either. His cases stay untouched (Standing Rule 38) and are excluded from our counts - we report "ours 475 / live 480". One of them (C38923) was RIGHT and exposed a real gap on our side, which we fixed on our own cases.</t>
+          <t>Not Chris's to give - the QA lead's / engineering's. Every observation on this sheet is PROVISIONAL until the branch is declared final (Standing Rule 49); the re-check queue is OPEN.</t>
         </is>
       </c>
       <c r="C146" s="6" t="inlineStr">
         <is>
-          <t>the 17-item sheet</t>
+          <t>the 10-row sheet</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="6" t="inlineStr">
         <is>
-          <t>The Technician Utilization column-selector story has no Jira ticket.</t>
+          <t>The 5 automated cases in our Report Suite folder authored by Vladimir Tomovic (C38919-C38923).</t>
         </is>
       </c>
       <c r="B147" s="6" t="inlineStr">
         <is>
-          <t>Ticket-management, not a product decision - he already asked for the control in his 2026-07-29 message ("for visual/natural conformance"), so scope is settled. TU-COL-01 (C38859) and TU-LOC-06 (C38915) cite epic SV-8582 and say so in refs. Tracked in OUTSTANDING-ITEMS-REGISTER.md as an OTHER TEAM item.</t>
+          <t>Not a Chris question, and by the QA lead's ruling 2026-07-31 we do not message Vladimir either. His cases stay untouched (Standing Rule 38) and are excluded from our counts - we report "ours 475 / live 480". One of them (C38923) was RIGHT and exposed a real gap on our side, which we fixed on our own cases.</t>
         </is>
       </c>
       <c r="C147" s="6" t="inlineStr">
@@ -4702,12 +4692,12 @@
     <row r="148">
       <c r="A148" s="6" t="inlineStr">
         <is>
-          <t>SV-8780 (the built dedicated Sales By Customer permission).</t>
+          <t>The Technician Utilization column-selector story has no Jira ticket.</t>
         </is>
       </c>
       <c r="B148" s="6" t="inlineStr">
         <is>
-          <t>OUT OF SCOPE by the QA lead's ruling 2026-08-03, verbatim: "Ignore this ticket." Not commented on, not transitioned, not read-and-edited. The drafted comment is retained unposted and banner-marked NOT TO BE POSTED.</t>
+          <t>Ticket-management, not a product decision - he already asked for the control in his 2026-07-29 message ("for visual/natural conformance"), so scope is settled. TU-COL-01 (C38859) and TU-LOC-06 (C38915) cite epic SV-8582 and say so in refs. Tracked in OUTSTANDING-ITEMS-REGISTER.md as an OTHER TEAM item.</t>
         </is>
       </c>
       <c r="C148" s="6" t="inlineStr">
@@ -4719,12 +4709,12 @@
     <row r="149">
       <c r="A149" s="6" t="inlineStr">
         <is>
-          <t>Four requirements we deliberately do not test (SBC S10-N1, SBR S11-N1, SBR S14-R14, PV S4-N1).</t>
+          <t>SV-8780 (the built dedicated Sales By Customer permission).</t>
         </is>
       </c>
       <c r="B149" s="6" t="inlineStr">
         <is>
-          <t>QA decisions, not product ones - cut by the user-authorized 2026-07-28 Ruthless Usefulness Audit as no-op assertions, un-measurable px font-tier minutiae, and a stored-schema state a manual tester cannot seed. Recorded with reasons in coverage-rederivation-2026-07-31/COVERAGE-REDERIVATION.md section 5.</t>
+          <t>OUT OF SCOPE by the QA lead's ruling 2026-08-03, verbatim: "Ignore this ticket." Not commented on, not transitioned, not read-and-edited. The drafted comment is retained unposted and banner-marked NOT TO BE POSTED.</t>
         </is>
       </c>
       <c r="C149" s="6" t="inlineStr">
@@ -4736,163 +4726,180 @@
     <row r="150">
       <c r="A150" s="6" t="inlineStr">
         <is>
+          <t>Four requirements we deliberately do not test (SBC S10-N1, SBR S11-N1, SBR S14-R14, PV S4-N1).</t>
+        </is>
+      </c>
+      <c r="B150" s="6" t="inlineStr">
+        <is>
+          <t>QA decisions, not product ones - cut by the user-authorized 2026-07-28 Ruthless Usefulness Audit as no-op assertions, un-measurable px font-tier minutiae, and a stored-schema state a manual tester cannot seed. Recorded with reasons in coverage-rederivation-2026-07-31/COVERAGE-REDERIVATION.md section 5.</t>
+        </is>
+      </c>
+      <c r="C150" s="6" t="inlineStr">
+        <is>
+          <t>the 17-item sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="6" t="inlineStr">
+        <is>
           <t>The QA branch / environment and fresh login cookies.</t>
         </is>
       </c>
-      <c r="B150" s="6" t="inlineStr">
+      <c r="B151" s="6" t="inlineStr">
         <is>
           <t>Not Chris's to give - this is the VIU blocker and it sits with the QA lead / engineering. All 475 cases remain VIU-Pending until it exists (Standing Rules 12/22).</t>
         </is>
       </c>
-      <c r="C150" s="6" t="inlineStr">
+      <c r="C151" s="6" t="inlineStr">
         <is>
           <t>the 17-item sheet</t>
         </is>
       </c>
     </row>
-    <row r="152">
-      <c r="A152" s="1" t="inlineStr">
+    <row r="153">
+      <c r="A153" s="1" t="inlineStr">
         <is>
           <t>LIVE EVIDENCE BEHIND TAB 1'S 'WHAT HAPPENS NOW' TEXT</t>
         </is>
       </c>
     </row>
-    <row r="153">
-      <c r="A153" s="3" t="inlineStr">
+    <row r="154">
+      <c r="A154" s="3" t="inlineStr">
         <is>
           <t>Observation</t>
         </is>
       </c>
-      <c r="B153" s="3" t="inlineStr">
+      <c r="B154" s="3" t="inlineStr">
         <is>
           <t>What was seen</t>
         </is>
       </c>
-      <c r="C153" s="3" t="inlineStr">
+      <c r="C154" s="3" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="D153" t="inlineStr"/>
-      <c r="E153" t="inlineStr"/>
-      <c r="F153" t="inlineStr"/>
-      <c r="G153" t="inlineStr"/>
-    </row>
-    <row r="154">
-      <c r="A154" s="6" t="inlineStr">
-        <is>
-          <t>Work In Progress, every location in view</t>
-        </is>
-      </c>
-      <c r="B154" s="6" t="inlineStr">
-        <is>
-          <t>Headers: WO # | Status | Customer | Asset | Advisor | Days Open | Earned | Remaining | Total. NO Location column. Location IS listed in the Column Selection panel.</t>
-        </is>
-      </c>
-      <c r="C154" s="6" t="inlineStr">
-        <is>
-          <t>evidence/location-behaviour.json; evidence/work-in-progress-selector.png</t>
-        </is>
-      </c>
+      <c r="D154" t="inlineStr"/>
+      <c r="E154" t="inlineStr"/>
+      <c r="F154" t="inlineStr"/>
+      <c r="G154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="6" t="inlineStr">
         <is>
-          <t>Work In Progress, one location in view</t>
+          <t>Work In Progress, every location in view</t>
         </is>
       </c>
       <c r="B155" s="6" t="inlineStr">
         <is>
-          <t>Identical headers - still no Location column.</t>
+          <t>Headers: WO # | Status | Customer | Asset | Advisor | Days Open | Earned | Remaining | Total. NO Location column. Location IS listed in the Column Selection panel.</t>
         </is>
       </c>
       <c r="C155" s="6" t="inlineStr">
         <is>
-          <t>evidence/location-single-vs-multi.json; evidence/wip-ONE-location-screen.png</t>
+          <t>evidence/location-behaviour.json; evidence/work-in-progress-selector.png</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="6" t="inlineStr">
         <is>
-          <t>Inventory Value, every location in view</t>
+          <t>Work In Progress, one location in view</t>
         </is>
       </c>
       <c r="B156" s="6" t="inlineStr">
         <is>
-          <t>Headers: Part # | Description | Category | Vendor | LOCATION | Qty | Unit Cost | Unit Sell | Margin | Margin % | Total Sell | Total Cost. Location present, and ALSO offered in the Column Selection panel.</t>
+          <t>Identical headers - still no Location column.</t>
         </is>
       </c>
       <c r="C156" s="6" t="inlineStr">
         <is>
-          <t>evidence/location-behaviour.json; evidence/inventory-value-selector.png</t>
+          <t>evidence/location-single-vs-multi.json; evidence/wip-ONE-location-screen.png</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="6" t="inlineStr">
         <is>
-          <t>Inventory Value, ONE location in view (the deviation)</t>
+          <t>Inventory Value, every location in view</t>
         </is>
       </c>
       <c r="B157" s="6" t="inlineStr">
         <is>
-          <t>Location filter reads 'Staging Lethbridge - 4310' (single) yet the Location column is STILL shown, every row repeating 'Staging Lethbridge - 4310'. Reproduced twice.</t>
+          <t>Headers: Part # | Description | Category | Vendor | LOCATION | Qty | Unit Cost | Unit Sell | Margin | Margin % | Total Sell | Total Cost. Location present, and ALSO offered in the Column Selection panel.</t>
         </is>
       </c>
       <c r="C157" s="6" t="inlineStr">
         <is>
-          <t>evidence/location-single-vs-multi.json; evidence/iv-ONE-location-screen.png</t>
+          <t>evidence/location-behaviour.json; evidence/inventory-value-selector.png</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="6" t="inlineStr">
         <is>
+          <t>Inventory Value, ONE location in view (the deviation)</t>
+        </is>
+      </c>
+      <c r="B158" s="6" t="inlineStr">
+        <is>
+          <t>Location filter reads 'Staging Lethbridge - 4310' (single) yet the Location column is STILL shown, every row repeating 'Staging Lethbridge - 4310'. Reproduced twice.</t>
+        </is>
+      </c>
+      <c r="C158" s="6" t="inlineStr">
+        <is>
+          <t>evidence/location-single-vs-multi.json; evidence/iv-ONE-location-screen.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="6" t="inlineStr">
+        <is>
           <t>Build marker (Standing Rule 49 - branch declared NOT FINAL)</t>
         </is>
       </c>
-      <c r="B158" s="6" t="inlineStr">
+      <c r="B159" s="6" t="inlineStr">
         <is>
           <t>v3.4.1-0ed4433 on sv8582.qa.shopview.com; index.html last-modified Mon, 03 Aug 2026 13:40:38 GMT, etag 02091e9dc11f187d7739b4efa166ea21 - byte-identical to the 2026-08-03 marker, so the build has not moved. All observations PROVISIONAL.</t>
         </is>
       </c>
-      <c r="C158" s="6" t="inlineStr">
+      <c r="C159" s="6" t="inlineStr">
         <is>
           <t>../viu-2026-08-03/RECHECK-QUEUE.md</t>
         </is>
       </c>
     </row>
-    <row r="160">
-      <c r="A160" s="1" t="inlineStr">
+    <row r="161">
+      <c r="A161" s="1" t="inlineStr">
         <is>
           <t>HONESTY NOTES</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="6" t="inlineStr">
-        <is>
-          <t>- Nothing here is rewritten. Every reader-facing row is the row its source sheet carried, emitted from that sheet's own generator, so the wording cannot drift in transit. The only text changes are the ones enumerated in the change log above.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="6" t="inlineStr">
         <is>
-          <t>- Standing Rule 49: the QA branch was declared NOT FINAL, so every build observation quoted on these tabs is PROVISIONAL and carries the build marker v3.4.1-0ed4433; the re-check queue viu-2026-08-03/RECHECK-QUEUE.md is OPEN.</t>
+          <t>- Nothing here is rewritten. Every reader-facing row is the row its source sheet carried, emitted from that sheet's own generator, so the wording cannot drift in transit. The only text changes are the ones enumerated in the change log above.</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="6" t="inlineStr">
         <is>
-          <t>- The Column Selection panel's per-item on/off state could not be read reliably by automation, so the "starts switched off" claim on Work In Progress rests on the column's absence from the grid plus the 2026-08-03 pass's own observation. The presence or absence of the column - which is what Tab 1's question turns on - is solid.</t>
+          <t>- Standing Rule 49: the QA branch was declared NOT FINAL, so every build observation quoted on these tabs is PROVISIONAL and carries the build marker v3.4.1-0ed4433; the re-check queue viu-2026-08-03/RECHECK-QUEUE.md is OPEN.</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="6" t="inlineStr">
+        <is>
+          <t>- The Column Selection panel's per-item on/off state could not be read reliably by automation, so the "starts switched off" claim on Work In Progress rests on the column's absence from the grid plus the 2026-08-03 pass's own observation. The presence or absence of the column - which is what Tab 1's question turns on - is solid.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="6" t="inlineStr">
         <is>
           <t>- Rule 37: the epic had a Tier-1 currency check only. A full re-read was not authorised for this pass and is not claimed.</t>
         </is>

</xml_diff>

<commit_message>
Consolidated Chris sheet: QA-only tab now spells out a TestRail link per case, per row
Standing Rule 8 asks for the internal ID + C-id + the /cases/view/<id> link on every row
that names a case. The first cut only spelled the links out for Tab 1's eight cases and
left the other rows with bare C-ids. Both QA tables (the per-item mapping and the
merged-out rows) now carry a "TestRail links" column derived from the C-ids in that row.

Verified on the produced workbook: 24 mapping rows, 0 rows that name a case without its
links; 93 C-id/link pairs, 0 where the number in the URL disagrees with its C-id; 102
link occurrences on the QA tab. Reader-facing gates unchanged - 0 findings on the .md and
all three reader-facing tabs; 102 internal-id/C-id pairs still verified against
testrail-id-map.csv.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
+++ b/build/report-suite/chris-consolidated-2026-08-04/Report-Suite_Questions-and-Decisions-for-Chris-Ward_2026-08-04.xlsx
@@ -1459,7 +1459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G165"/>
+  <dimension ref="A1:H165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1467,8 +1467,9 @@
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="56" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
     <col width="56" customWidth="1" min="7" max="7"/>
+    <col width="56" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1520,10 +1521,15 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
+          <t>TestRail links</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
           <t>Spec anchors + live evidence</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>What each answer resolves to</t>
         </is>
@@ -1557,10 +1563,15 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
+          <t>C30551 https://shopview.testrail.io/index.php?/cases/view/30551 · C30554 https://shopview.testrail.io/index.php?/cases/view/30554 · C30580 https://shopview.testrail.io/index.php?/cases/view/30580 · C30588 https://shopview.testrail.io/index.php?/cases/view/30588 · C38917 https://shopview.testrail.io/index.php?/cases/view/38917 · C30466 https://shopview.testrail.io/index.php?/cases/view/30466 · C30467 https://shopview.testrail.io/index.php?/cases/view/30467 · C38916 https://shopview.testrail.io/index.php?/cases/view/38916</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
           <t>Inventory Value spec v3 S7-R6; WIP spec v6 S4-R3; S7-R13</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>If Chris answers A (automatic - matches both specs): All 8 cases are re-worded to assert the automatic, scope-driven model that SBC/SBR/PV/TU already use, and the observed selector-controlled build is recorded as a DEVIATION in the case notes (the pattern WIP-FLT-05 = C30502 already uses). Two build defects get raised: Work In Progress never shows it automatically; Inventory Value never hides it at single scope on screen. This is the outcome Standing Rule 33 already points to - the specs outrank our build observation - so A costs 8 re-words and 2 tickets. || If Chris answers B (user-toggled): All 8 cases stand exactly as they are; no TestRail write is needed. Chris updates the two written descriptions (WIP S4-R3 + S7-R13, IV S7-R6). The 11 cases on the other four reports that assert the automatic model stay correct, because B would apply only to the two reports whose descriptions change - CONFIRM THIS WITH HIM if he picks B, since a suite-wide B would invalidate those 11. || If Chris answers C (something else / differs per report): Re-derive per report from his answer; expect a further reconciliation pass and treat all 8 as blocked until then. || Regardless of the answer - a separate surface split to settle: On Inventory Value the SCREEN keeps the Location column at single scope while the CSV download drops it (screen observed 2026-08-04; CSV observed 2026-08-03, viu-2026-08-03/evidence/location-matrix/inventory-value__SINGLE__plain.csv has no Location header, __MULTI__ does). Two surfaces, two behaviours - IV-EXP-02 (C30588) is the export case affected. Standing Rule 40: every surface gets its own verdict.</t>
         </is>
@@ -1594,10 +1605,15 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
+          <t>C30216 https://shopview.testrail.io/index.php?/cases/view/30216 · C30340 https://shopview.testrail.io/index.php?/cases/view/30340 · C30446 https://shopview.testrail.io/index.php?/cases/view/30446 · C30503 https://shopview.testrail.io/index.php?/cases/view/30503 · C30577 https://shopview.testrail.io/index.php?/cases/view/30577 · C30109 https://shopview.testrail.io/index.php?/cases/view/30109</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
           <t>OUR SOURCE: Chris Ward 2026-07-31 Q1=A, verbatim "A -- classic spec drift" (chris-answers-2026-07-31/answers-ingested.md). THE BUILD'S SOURCE: SBR v15 S21-N1, PV v4 S2-E4, TU v5 S9-N1, IV v3 S7-N1 - all four still read "still sees the filter". LIVE: viu-2026-08-03/evidence/singleloc-matrix.json - hasLocationControl TRUE on all six for the single-workplace subject; build v3.4.1-0ed4433. Verdicts: batch-sbc-sbr/VERDICTS.md SBR-LOC-04, batch-pv-tu/VERDICTS.md PV-FILT-13 + TU-LOC-05, batch-wip-iv/VERDICTS.md IV-LOC-04. RECHECK-QUEUE row B18 (flagged there as the single most important row to re-check).</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>A -&gt; the 5 cases flip from 'filter hidden' to 'filter shown', and SBC needs no new case. B -&gt; no case change; a dev ticket is raised for all six, and SBC needs a NEW case for parity. Either way the four spec notes need his edit. All 5 currently sit DEVIATION and are HELD (batch-wip-iv/STAGED-CHANGES.md group C2) - deliberately not edited, because editing them would assert behaviour no written source supports.</t>
         </is>
@@ -1631,10 +1647,15 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
+          <t>C30470 https://shopview.testrail.io/index.php?/cases/view/30470 · C30485 https://shopview.testrail.io/index.php?/cases/view/30485 · C30500 https://shopview.testrail.io/index.php?/cases/view/30500 · C30516 https://shopview.testrail.io/index.php?/cases/view/30516 · C30134 https://shopview.testrail.io/index.php?/cases/view/30134</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
           <t>OUR SOURCE: Chris Ward 2026-07-29, verbatim "A is the correct answer" plus the durable instruction "Not just for these specs though -- really good to keep this in mind for all actions moving forward" (chris-update-2026-07-29/wip-identifier-answer-2026-07-29.md). THE BUILD'S SOURCE: WIP v6 S4-R7 ("the unit number on the first line in bold, and the vehicle identification number on the second line") and S4-R9 ("The Asset column sorts by unit number"). LIVE DOM, verbatim: &lt;div class="wip-asset"&gt;&lt;span class="wip-asset__unit text-weight-bold"&gt;6548&lt;/span&gt;&lt;span class="wip-asset__vin text-caption text-grey-7"&gt;1FDSE3EL1EDB20609&lt;/span&gt;&lt;/div&gt;. Serial-style values live in the VIN field: BULK PARTS1, 12-06696, P631627, 86J8FAC1VALJ43SJY. Build v3.4.1-0ed4433. HONEST LIMIT: we did not CREATE a non-vehicle asset - the report has no asset-creation surface; the terminology point is evidenced from existing records only (batch-wip-iv/STAGED-CHANGES.md group C1).</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>A -&gt; dev ticket; the 4 cases stand as written and he edits S4-R7/S4-R9. B -&gt; the 4 cases revert to unit-number-leads and the durable CLAUDE.md ruling is narrowed to exclude this report. C -&gt; a label change is a new question for the whole suite, including SBC-LBL-01. All 4 are HELD, not edited.</t>
         </is>
@@ -1668,10 +1689,15 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
+          <t>C30285 https://shopview.testrail.io/index.php?/cases/view/30285 · C30286 https://shopview.testrail.io/index.php?/cases/view/30286</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
           <t>Three sources, three words. SPEC: SBR v15 S14-R15/S14-R16 both open with `Sales Rep`. OUR SOURCE: Chris Ward 2026-07-31 Q5=A, verbatim "Rep is too much slang, let's do representative everywhere" - so our cases correctly say "Sales Representative" (Rule 32). BUILD: header line read from evidence/location-matrix/sales-by-representative__SINGLE__summary.csv line 2 = `Representative,"Inv. Hrs",...`; the expanded file agrees. Build v3.4.1-0ed4433. Analysis: viu-2026-08-03/LABEL-DIFF.md section A4, which explicitly says do NOT edit these two to "Representative" before he rules.</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>A -&gt; both cases reworded to "Representative" and he tidies S14-R15/R16. B -&gt; dev ticket; the cases stand. Either way these two cases also carry item 5 (the four missing columns) and the separate LABEL-DIFF A6 findings (the expanded file puts Invoice # before Date and heads the status column "Invoice Status"), so all of it lands as ONE combined edit per case, each re-verified WHOLE against the current spec per Rule 41.</t>
         </is>
@@ -1705,10 +1731,15 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
+          <t>C30285 https://shopview.testrail.io/index.php?/cases/view/30285</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
           <t>SPEC (Rule 25, verbatim): SBR v15 S14-R15 "Headers, in order: `Sales Rep`, `# Invoices`, `# Customers`, `Hrs Worked`, `Hrs Invoiced`, `Inv. Hrs`, `Labor Invoiced`, `Labor Margin`, `Parts Invoiced`, `Parts Margin`, `Margin`, `Margin %`, `Subtotal`." = 13. BUILD: 9 - `Representative, Inv. Hrs, Labor Invoiced, Labor Margin, Parts Invoiced, Parts Margin, Margin, Margin %, Subtotal` (evidence/location-matrix/sales-by-representative__SINGLE__summary.csv). Missing: # Invoices, # Customers, Hrs Worked, Hrs Invoiced. The payload DOES carry invoice_count, hours_worked and hours_invoiced, which is why LABEL-DIFF.md A5 reads it as an unfinished export, not a data defect. Build v3.4.1-0ed4433. NOTE: S14-R16 itself carries a build note asking engineering to align the hours columns, so his own document already half-anticipates this.</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>A -&gt; dev ticket; C30285 stands as written. B -&gt; C30285's enumeration shortens to nine and he shortens S14-R15. Rule 42 applies either way: the rewritten enumeration must carry a version-pinned anchor.</t>
         </is>
@@ -1742,10 +1773,15 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
+          <t>C30102 https://shopview.testrail.io/index.php?/cases/view/30102 · C30104 https://shopview.testrail.io/index.php?/cases/view/30104 · C30201 https://shopview.testrail.io/index.php?/cases/view/30201 · C30330 https://shopview.testrail.io/index.php?/cases/view/30330 · C30501 https://shopview.testrail.io/index.php?/cases/view/30501 · C30561 https://shopview.testrail.io/index.php?/cases/view/30561</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
           <t>SPEC: SBC v13 S2-R2 closes the eleven-item list verbatim; WIP v6 S7-R6 and IV v3 S5-R1 close the same list in their own words. BUILD: nine presets + inline calendar + "Range: N days" + Apply, captured verbatim in viu-2026-08-03/evidence/date-range-picker.json. Build v3.4.1-0ed4433. This is the application's SHARED date component, so it is a suite-wide product decision. Registered as DELIBERATE-DECISIONS.md entry 2.1 at risk MEDIUM precisely because C30104's steps cannot be executed today.</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>A -&gt; 6 cases reworded to the nine presets + calendar, C30104 becomes runnable, and 3 specs need his edit. B -&gt; dev ticket against the shared component; all 6 cases stand and C30104 stays unrunnable until it ships. C -&gt; partial dev ticket plus a partial case rewrite.</t>
         </is>
@@ -1779,10 +1815,15 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
+          <t>C30434 https://shopview.testrail.io/index.php?/cases/view/30434 · C30435 https://shopview.testrail.io/index.php?/cases/view/30435</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
           <t>SPEC (Rule 25, verbatim): TU v5 S7-R2 'an option labeled "Download Summary (PDF)"', S7-R3 '"Download Expanded View (PDF)"', S7-R4 '"Download (CSV)"' = three items with the Download prefix. BUILD: four items - `Summary (PDF)`, `Summary (CSV)`, `Expanded (PDF)`, `Expanded (CSV)`, no prefix (batch-pv-tu/VERDICTS.md TU-EXP-01; evidence/tu/ui/tu-ui-*.json). CONTRAST captured the same run: SBC and SBR both show the four long labels and MATCH their specs exactly (batch-sbc-sbr/VERDICTS.md F2, LABEL-DIFF.md B row SBC-EXP-01). Build v3.4.1-0ed4433. Registered as DELIBERATE-DECISIONS.md entry 2.4, risk MEDIUM.</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>A -&gt; C30434 reworded to the four shipped strings (and C30435's Summary-PDF scope re-checked), and he edits S7-R2/R3/R4 to four items. B -&gt; dev ticket; both cases stand.</t>
         </is>
@@ -1816,10 +1857,15 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
+          <t>C30590 https://shopview.testrail.io/index.php?/cases/view/30590</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
           <t>SPEC (Rule 25, verbatim): IV v3 S10-R8 "The PDF header shows the report name 'Inventory Value', the organization name, the selected period, and an 'as of' line naming the day the values represent..." - the PDF only; no requirement mentions the CSV. S10-R15 governs only the "Locations:" line. BUILD: CSV line 1 = "As of: 2026-08-03" with the locations line on line 2 (evidence/location-matrix/inventory-value__SINGLE__plain.csv); extracted PDF header block reads `As of 2026-08-04` with NO colon (batch-wip-iv/STAGED-CHANGES.md B28). Build v3.4.1-0ed4433. This surfaced from the SURFACE-MATRIX 1b sweep (Rule 40) - the IV "Locations:" line is the only one of six that is line 2 rather than line 1, because the as-of line sits above it.</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>A -&gt; he adds the CSV as-of line to S10-R8 (or a new requirement) and C30590 gains the CSV half. B -&gt; dev ticket to remove it; C30590 unchanged. C -&gt; a wording ticket plus a one-line spec edit; C30590 quotes whichever string he picks.</t>
         </is>
@@ -1853,10 +1899,15 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
+          <t>C30325 https://shopview.testrail.io/index.php?/cases/view/30325 · C30327 https://shopview.testrail.io/index.php?/cases/view/30327 · C30391 https://shopview.testrail.io/index.php?/cases/view/30391 · C30398 https://shopview.testrail.io/index.php?/cases/view/30398 · C30526 https://shopview.testrail.io/index.php?/cases/view/30526 · C30527 https://shopview.testrail.io/index.php?/cases/view/30527 · C30603 https://shopview.testrail.io/index.php?/cases/view/30603 · C30604 https://shopview.testrail.io/index.php?/cases/view/30604</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
           <t>ALREADY RULED - no product decision is being re-asked. Chris Ward 2026-07-31 Q4=A, verbatim "A - the intention is to not hide these from normal reports access. These were specced before CRP was built :)" (and the same answer 2026-07-28), plus the QA LEAD's ruling 2026-08-03, verbatim: "Yes all the reports will be gated by ONE permission FOR NOW." SPEC TEXT STILL STALE: PV v4 S1-R4 + S1-N2, IV v3 Story-1 prerequisite, TU v5 Story-1 prerequisite, WIP v6 Story-1 prerequisite; SBC v13 S1-R2 has been corrected. LIVE PROOF BOTH WAYS (viu-2026-08-03/SURFACE-MATRIX.md Matrix 2 + evidence/permissions/permission-matrix.json + minimal-role-proof.json): the FE permission catalogue holds exactly one report atom; an 8-atom Sales Representative holding only it got 200 on data AND export for all six; a Foreman without it got 403 on all six, data and export. Build v3.4.1-0ed4433. This is why C30327 and C30391 are verified MORE strongly than written - the extra per-report permission does not merely fail to enforce, it does not exist.</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>No case change on any answer - all 8 already follow the ruling. This row only closes a documentation debt on four spec pages. The separate rescope-or-retire decision on C30327 and C30391 is the QA LEAD's, not Chris's (chris-answers-2026-08-01/staged-case-plan-CDE-2026-08-03.md).</t>
         </is>
@@ -1890,10 +1941,15 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
+          <t>C30159 https://shopview.testrail.io/index.php?/cases/view/30159 · C30172 https://shopview.testrail.io/index.php?/cases/view/30172</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
           <t>SPEC: SBC v13 S18-R7 "Exports (CSV, PDF, Print) are generated on the server..." and S18-R10 "If an export (CSV, PDF, or Print) is triggered while the active filters match no customers..." - both still name Print, although Chris retired it in Story 16 ("(removed - Print retired)"). JIRA SV-8614 "SBC - Story 16 - Print the report" is still OPEN. BUILD: a sweep of every button, menu item and link for 'print' in text or aria-label returned an EMPTY list on all six reports (batch-sbc-sbr/VERDICTS.md F3; evidence/sales-by-customer/observe-full.json#toolbar.printControls). Build v3.4.1-0ed4433. Registered as DELIBERATE-DECISIONS.md entry 1.4 at risk LOW, and as an OUTSIDE-IN.md external signal.</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>No decision and no case change - C30159 explicitly asserts the ABSENCE of Print and PASSED live. Included only so a documentation tidy-up and the closure of SV-8614 are not forgotten; SV-8614 is a dev/ticket action, not Chris's.</t>
         </is>
@@ -1927,10 +1983,15 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
+          <t>C30285 https://shopview.testrail.io/index.php?/cases/view/30285 · C30286 https://shopview.testrail.io/index.php?/cases/view/30286 · C30278 https://shopview.testrail.io/index.php?/cases/view/30278 · C30279 https://shopview.testrail.io/index.php?/cases/view/30279 · C38913 https://shopview.testrail.io/index.php?/cases/view/38913</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
           <t>SBR spec v15 (Confluence 585629698, lastModified 2026-07-29 - RE-VERIFIED LIVE 2026-08-03, still unresolved): NEW S14-R20 ("included in all four exports in the same position it occupies on screen") vs S14-R15 (Summary CSV headers "in order", beginning `Sales Rep`, no Location) and S14-R16 (Expanded CSV headers). The header enumerations date from the 2026-07-11 "Exports hardened" round and were never amended. Corroborated by contradiction-analysis-2026-07-31/SBR-CSV-LOCATION.md and by Vladimir Tomovic's automated C38923, which was RIGHT (Rule 44).</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>A -&gt; the 5 cases stand as pushed and Chris tidies S14-R15/R16. B -&gt; revert the export halves to the fixed lists and drop the Location assertions. Same on-screen/export split was fixed on SBC (S4-R13), PV (S6-R11), TU (S7-R13), IV (S10-R15); WIP already had it. Either way VIU-confirm live.</t>
         </is>
@@ -1964,10 +2025,15 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
+          <t>C30470 https://shopview.testrail.io/index.php?/cases/view/30470 · C30500 https://shopview.testrail.io/index.php?/cases/view/30500 · C30485 https://shopview.testrail.io/index.php?/cases/view/30485 · C30516 https://shopview.testrail.io/index.php?/cases/view/30516 · C30216 https://shopview.testrail.io/index.php?/cases/view/30216 · C30446 https://shopview.testrail.io/index.php?/cases/view/30446 · C30577 https://shopview.testrail.io/index.php?/cases/view/30577 · C30340 https://shopview.testrail.io/index.php?/cases/view/30340 · C30392 https://shopview.testrail.io/index.php?/cases/view/30392 · C30322 https://shopview.testrail.io/index.php?/cases/view/30322</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
           <t>SPEC-WATCH-2026-07-28.md re-diff 2026-07-31, re-confirmed 2026-08-03 (all five non-SBC specs still at their 2026-07-29 versions per live CQL, so nothing has landed since): 7 of 12 items still need spec text - 1b WIP identifier, 4 location filter hidden, 6 nav placement wording, 8 WIP asset dropdown, 9 customer-card Representative, 10 SBC nav anchors, 11 PV "only report". Deadline 2026-08-04.</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>A -&gt; no case change; SPEC-WATCH stays open until the text lands. B -&gt; SPEC-WATCH closes as a documentation debt. Neither answer changes a case. Items 1b/4/6/9/10/11 are ALSO asked individually as sheet items 6-12 so he can tick them off.</t>
         </is>
@@ -2001,10 +2067,15 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
+          <t>C38856 https://shopview.testrail.io/index.php?/cases/view/38856 · C38912 https://shopview.testrail.io/index.php?/cases/view/38912 · C30285 https://shopview.testrail.io/index.php?/cases/view/30285 · C30278 https://shopview.testrail.io/index.php?/cases/view/30278 · C38913 https://shopview.testrail.io/index.php?/cases/view/38913</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
           <t>SPEC-SILENT, found by coverage-rederivation-2026-07-31. SBC S4-R13 states inclusion with no position; SBR S14-R20 says "the same position it occupies on screen" but the Summary CSV (S14-R15) has no Date/Status column and the Summary PDF (S14-R5) has none either. Cases currently hedge ("with the identifying columns ahead of the money columns (confirm its exact position in the build)") - hedged, not invented (Rule 9).</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>A -&gt; replace the hedge with the stated position. B -&gt; reword to far-right. C -&gt; keep the hedge and pin it at VIU. No case is wrong today either way.</t>
         </is>
@@ -2038,10 +2109,15 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
+          <t>C30168 https://shopview.testrail.io/index.php?/cases/view/30168 · C30439 https://shopview.testrail.io/index.php?/cases/view/30439 · C30440 https://shopview.testrail.io/index.php?/cases/view/30440 · C30379 https://shopview.testrail.io/index.php?/cases/view/30379 · C30380 https://shopview.testrail.io/index.php?/cases/view/30380 · C30278 https://shopview.testrail.io/index.php?/cases/view/30278 · C30279 https://shopview.testrail.io/index.php?/cases/view/30279</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
           <t>Cross-report spec contradiction against his 2026-07-29 message ("Each report now ensures the same 'logo' treatment"): SBC S15-R16/R17/R18 = 3-step chain ending in NO logo; TU = bundled ShopView default; PV has no logo requirement at all. DELIBERATE-DECISIONS.md A2. Not resolved by us (Rule 15 - never pick a side silently).</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>A -&gt; TU/PV export cases gain the fallback chain. B -&gt; SBC-EXP-10's chain collapses to the bundled default. C -&gt; re-ask. Wording-only edits either way.</t>
         </is>
@@ -2075,10 +2151,15 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
+          <t>C30102 https://shopview.testrail.io/index.php?/cases/view/30102</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
           <t>His chat, verbatim: "SBC actually has several features that we dropped almost right before the squad assembled ... the requirements should have dropped with the additional features dropping, I own that." Checked live 2026-08-03 against the SBC spec change log (Confluence 577634305): the four dropped rounds are 2026-07-12 (customer comparison + asset comparison), 2026-07-15 (global search), 2026-07-16 (All Time), 2026-07-29 (Print). ZERO lingering requirements and ZERO stale cases found - see chris-answers-2026-08-01/answers-ingested.md section 3.</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>A -&gt; the item closes with a written all-clear. B -&gt; re-derive coverage for whatever he names. We did NOT manufacture a retire list to fill the gap (Rule 12).</t>
         </is>
@@ -2110,12 +2191,13 @@
           <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off ["row 2" here means the source sheet's own item-2 mapping row, which is Tab 3 item 2 above]</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr"/>
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>Named individually at the QA lead's instruction ("each named individually, not as a bundle"), because the 2026-08-04 deadline is tomorrow and a bundled question has so far produced a bundled non-answer. [this mapping row covers items 6-12 of the source sheet; after the de-duplication its surviving items are Tab 3 items 6, 7, 8, 9, 10]</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>No case change on any answer - the cases already follow his rulings (Rule 32). These only close a documentation debt.</t>
         </is>
@@ -2147,12 +2229,13 @@
           <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off ["row 2" here means the source sheet's own item-2 mapping row, which is Tab 3 item 2 above]</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr"/>
+      <c r="G22" s="6" t="inlineStr">
         <is>
           <t>Named individually at the QA lead's instruction ("each named individually, not as a bundle"), because the 2026-08-04 deadline is tomorrow and a bundled question has so far produced a bundled non-answer. [this mapping row covers items 6-12 of the source sheet; after the de-duplication its surviving items are Tab 3 items 6, 7, 8, 9, 10]</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>No case change on any answer - the cases already follow his rulings (Rule 32). These only close a documentation debt.</t>
         </is>
@@ -2184,12 +2267,13 @@
           <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off ["row 2" here means the source sheet's own item-2 mapping row, which is Tab 3 item 2 above]</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr"/>
+      <c r="G23" s="6" t="inlineStr">
         <is>
           <t>Named individually at the QA lead's instruction ("each named individually, not as a bundle"), because the 2026-08-04 deadline is tomorrow and a bundled question has so far produced a bundled non-answer. [this mapping row covers items 6-12 of the source sheet; after the de-duplication its surviving items are Tab 3 items 6, 7, 8, 9, 10]</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>No case change on any answer - the cases already follow his rulings (Rule 32). These only close a documentation debt.</t>
         </is>
@@ -2221,12 +2305,13 @@
           <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off ["row 2" here means the source sheet's own item-2 mapping row, which is Tab 3 item 2 above]</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>Named individually at the QA lead's instruction ("each named individually, not as a bundle"), because the 2026-08-04 deadline is tomorrow and a bundled question has so far produced a bundled non-answer. [this mapping row covers items 6-12 of the source sheet; after the de-duplication its surviving items are Tab 3 items 6, 7, 8, 9, 10]</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>No case change on any answer - the cases already follow his rulings (Rule 32). These only close a documentation debt.</t>
         </is>
@@ -2258,12 +2343,13 @@
           <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off ["row 2" here means the source sheet's own item-2 mapping row, which is Tab 3 item 2 above]</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr"/>
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>Named individually at the QA lead's instruction ("each named individually, not as a bundle"), because the 2026-08-04 deadline is tomorrow and a bundled question has so far produced a bundled non-answer. [this mapping row covers items 6-12 of the source sheet; after the de-duplication its surviving items are Tab 3 items 6, 7, 8, 9, 10]</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>No case change on any answer - the cases already follow his rulings (Rule 32). These only close a documentation debt.</t>
         </is>
@@ -2297,10 +2383,15 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
+          <t>C30255 https://shopview.testrail.io/index.php?/cases/view/30255</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
           <t>ANSWERED by Chris 2026-07-28, verbatim "B." (chris-answers-2026-07-28/answers-ingested.md Q1) = Escape must NOT dismiss. Verified live 2026-08-03: SBR S13-R8 still says Escape closes the dialog. NOTE - a correction to our own record: PO-Questions-Chris-ReportSuite-2026-07-31.md line 125 says this question is still "open four days". That is STALE; only the spec text remains outstanding, which is why this appears here as a write-down item, not a decision.</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>No case change - C30255 already follows his answer.</t>
         </is>
@@ -2334,10 +2425,15 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
+          <t>C38885 https://shopview.testrail.io/index.php?/cases/view/38885 · C38887 https://shopview.testrail.io/index.php?/cases/view/38887 · C38918 https://shopview.testrail.io/index.php?/cases/view/38918</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
           <t>His 2026-07-31 Q2=A ("A - great catch", one suite-wide message) + Q3=A ("this was not well thought out by me", cap on all six). Verified: the PV/TU/WIP pages carry no cap line; the three cases exist and are pushed.</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>No case change - documentation debt only.</t>
         </is>
@@ -2371,10 +2467,15 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
+          <t>C30134 https://shopview.testrail.io/index.php?/cases/view/30134 · C30470 https://shopview.testrail.io/index.php?/cases/view/30470</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
           <t>His own 2026-07-29 standing note, verbatim: "we just have to be careful with using the acronym VIN ... for a generator ... it gets confusing". Our cases keep the build label "VIN" plus a plain tester note, per the durable ruling in CLAUDE.md.</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>No case change either way - the on-screen label is unaffected.</t>
         </is>
@@ -2406,12 +2507,13 @@
           <t>NONE</t>
         </is>
       </c>
-      <c r="F29" s="6" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr"/>
+      <c r="G29" s="6" t="inlineStr">
         <is>
           <t>Cosmetic encoding artefact (mojibake) in the SBR and PV spec text, already noted in SPEC-WATCH-2026-07-28.md. Not a product question; asked only because it makes quoting those lines back to him unreliable.</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>No case impact.</t>
         </is>
@@ -2456,6 +2558,7 @@
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -2744,6 +2847,7 @@
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -2863,15 +2967,20 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
+          <t>TestRail links</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
           <t>Spec anchors + live evidence</t>
         </is>
       </c>
-      <c r="F50" s="3" t="inlineStr">
+      <c r="G50" s="3" t="inlineStr">
         <is>
           <t>What each answer resolves to</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
@@ -2896,10 +3005,15 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
+          <t>C30467 https://shopview.testrail.io/index.php?/cases/view/30467 · C30466 https://shopview.testrail.io/index.php?/cases/view/30466 · C30507 https://shopview.testrail.io/index.php?/cases/view/30507 · C38916 https://shopview.testrail.io/index.php?/cases/view/38916 · C38917 https://shopview.testrail.io/index.php?/cases/view/38917 · C30554 https://shopview.testrail.io/index.php?/cases/view/30554</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
           <t>SPEC: WIP v6 S4-R3 + S7-R13 ("not offered in the column selector; its visibility is automatic"); IV v3 Story-7 context note + S7-R7 ("not a user-toggled column in the column-selection control"). LIVE: viu-2026-08-03/batch-wip-iv/evidence/ui/colsel-work-in-progress.json - Location is item index 5 of 16, ariaChecked=false; colsel-inventory-value.json - Location is item index 4 of 11, ariaChecked=true; iv-singleloc.png shows the column still present with the chooser narrowed to Staging Lethbridge - 4310. Build v3.4.1-0ed4433. ALSO OUR OWN CONTRADICTION (Rule 28 cross-case sweep): C30466 and C30507 both list Location inside the toggleable order while C30467 says it is not offered - that self-contradiction is resolved whichever way he rules. HONEST LIMIT: the separate one-location-USER read of the IV screen was CONFOUNDED by a persisted column selection (RECHECK-QUEUE B34, recorded NOT VERIFIED); the observation quoted to Chris is the ADMIN-NARROWING one, which is clean. Note also that the IV single-location CSV has NO Location column (evidence/location-matrix/inventory-value__SINGLE__plain.csv), so the download already follows the automatic rule while the screen follows the toggle.</t>
         </is>
       </c>
-      <c r="F51" s="6" t="inlineStr">
+      <c r="G51" s="6" t="inlineStr">
         <is>
           <t>A -&gt; dev ticket for both reports; the 6 cases stand as written and the two specs need no change. B -&gt; both specs need his edit and the 6 cases are reworded to the toggle model (WIP off-by-default, IV on-by-default, or one agreed default). C -&gt; the two reports are documented as deliberately different and our cross-case contradiction is closed by writing each report's own model down.</t>
         </is>
@@ -2926,12 +3040,13 @@
           <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off [this is the grouped mapping row the source sheet used for its items 6-12; "row 2" in its text means the sheet's own item-2 row, which is carried above as Tab 3 item 2]</t>
         </is>
       </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="E52" s="6" t="inlineStr"/>
+      <c r="F52" s="6" t="inlineStr">
         <is>
           <t>Named individually at the QA lead's instruction ("each named individually, not as a bundle"), because the 2026-08-04 deadline is tomorrow and a bundled question has so far produced a bundled non-answer.</t>
         </is>
       </c>
-      <c r="F52" s="6" t="inlineStr">
+      <c r="G52" s="6" t="inlineStr">
         <is>
           <t>No case change on any answer - the cases already follow his rulings (Rule 32). These only close a documentation debt.</t>
         </is>
@@ -2958,12 +3073,13 @@
           <t>Same cases as row 2 - these are SPEC-WATCH items 1b, 4, 6, 10, 8, 9, 11 asked one at a time so he can tick each off [this is the grouped mapping row the source sheet used for its items 6-12; "row 2" in its text means the sheet's own item-2 row, which is carried above as Tab 3 item 2]</t>
         </is>
       </c>
-      <c r="E53" s="6" t="inlineStr">
+      <c r="E53" s="6" t="inlineStr"/>
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>Named individually at the QA lead's instruction ("each named individually, not as a bundle"), because the 2026-08-04 deadline is tomorrow and a bundled question has so far produced a bundled non-answer.</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr">
+      <c r="G53" s="6" t="inlineStr">
         <is>
           <t>No case change on any answer - the cases already follow his rulings (Rule 32). These only close a documentation debt.</t>
         </is>
@@ -2992,10 +3108,15 @@
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
+          <t>C30325 https://shopview.testrail.io/index.php?/cases/view/30325 · C30327 https://shopview.testrail.io/index.php?/cases/view/30327 · C30391 https://shopview.testrail.io/index.php?/cases/view/30391 · C30603 https://shopview.testrail.io/index.php?/cases/view/30603 · C30604 https://shopview.testrail.io/index.php?/cases/view/30604 · C30398 https://shopview.testrail.io/index.php?/cases/view/30398 · C30526 https://shopview.testrail.io/index.php?/cases/view/30526 · C30527 https://shopview.testrail.io/index.php?/cases/view/30527 · C30322 https://shopview.testrail.io/index.php?/cases/view/30322 · C30534 https://shopview.testrail.io/index.php?/cases/view/30534 · C30392 https://shopview.testrail.io/index.php?/cases/view/30392 · C30451 https://shopview.testrail.io/index.php?/cases/view/30451</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
           <t>NEW spec debt created by his own Q2=A ("Collapse all report access into a single Reports permission") plus the QA lead's ruling 2026-08-03, verbatim: "Yes all the reports will be gated by ONE permission FOR NOW." Verified live 2026-08-03: PV S1-R4/S1-N2, IV S1-R4 and the TU/WIP Story-1 prerequisites still name per-area permissions; only SBC S1-R2 has been corrected (2026-07-31). NOTE: the SBC change log still instructs engineering to DROP the atom, while his later chat allows hiding it inert - the later source wins (Rule 32).</t>
         </is>
       </c>
-      <c r="F54" s="6" t="inlineStr">
+      <c r="G54" s="6" t="inlineStr">
         <is>
           <t>No decision needed - the model is settled. Groups C and D of staged-case-plan-CDE-2026-08-03.md reword these 12 cases to the single permission; the two retire-or-rescope candidates (C30327, C30391) await the QA lead's sign-off.</t>
         </is>
@@ -3028,6 +3149,7 @@
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
@@ -3175,6 +3297,7 @@
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
@@ -3228,6 +3351,7 @@
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
@@ -3598,6 +3722,7 @@
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="6" t="inlineStr">
@@ -4286,6 +4411,7 @@
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr"/>
+      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="6" t="inlineStr">
@@ -4518,6 +4644,7 @@
       <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
@@ -4784,6 +4911,7 @@
       <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr"/>
+      <c r="H154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="6" t="inlineStr">

</xml_diff>